<commit_message>
Added year to GREET data
</commit_message>
<xml_diff>
--- a/data/MetCouncilTables.xlsx
+++ b/data/MetCouncilTables.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://icfonline-my.sharepoint.com/personal/61886_icf_com/Documents/Desktop/transport-emission-shiny/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{BBC49CD7-68E0-4D8F-B576-EE14E509F0DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="25" documentId="8_{BBC49CD7-68E0-4D8F-B576-EE14E509F0DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9A42A5A0-4EEB-4C5D-A128-675A4F344D14}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="14" activeTab="18" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView minimized="1" xWindow="345" yWindow="675" windowWidth="27645" windowHeight="15150" firstSheet="1" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ProjectTypes" sheetId="1" r:id="rId1"/>
@@ -51,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="450" uniqueCount="199">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="507" uniqueCount="200">
   <si>
     <t>category</t>
   </si>
@@ -648,13 +648,16 @@
   </si>
   <si>
     <t>N2O</t>
+  </si>
+  <si>
+    <t>Year</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -666,6 +669,13 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF181818"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -691,7 +701,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -699,6 +709,7 @@
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -5473,40 +5484,1226 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:G58"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="21.28515625" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>199</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>2024</v>
+      </c>
+      <c r="B2" t="s">
         <v>49</v>
       </c>
-      <c r="B2">
+      <c r="C2">
         <v>409.73</v>
       </c>
-      <c r="C2">
+      <c r="D2">
         <v>342.66</v>
       </c>
-      <c r="D2">
+      <c r="E2">
         <v>355.23</v>
       </c>
-      <c r="E2">
+      <c r="F2">
+        <v>175.45</v>
+      </c>
+      <c r="G2" s="5"/>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <f>A2+1</f>
+        <v>2025</v>
+      </c>
+      <c r="B3" t="s">
+        <v>49</v>
+      </c>
+      <c r="C3">
+        <v>409.73</v>
+      </c>
+      <c r="D3">
+        <v>342.66</v>
+      </c>
+      <c r="E3">
+        <v>355.23</v>
+      </c>
+      <c r="F3">
+        <v>175.45</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <f t="shared" ref="A4:A58" si="0">A3+1</f>
+        <v>2026</v>
+      </c>
+      <c r="B4" t="s">
+        <v>49</v>
+      </c>
+      <c r="C4">
+        <v>409.73</v>
+      </c>
+      <c r="D4">
+        <v>342.66</v>
+      </c>
+      <c r="E4">
+        <v>355.23</v>
+      </c>
+      <c r="F4">
+        <v>175.45</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <f t="shared" si="0"/>
+        <v>2027</v>
+      </c>
+      <c r="B5" t="s">
+        <v>49</v>
+      </c>
+      <c r="C5">
+        <v>409.73</v>
+      </c>
+      <c r="D5">
+        <v>342.66</v>
+      </c>
+      <c r="E5">
+        <v>355.23</v>
+      </c>
+      <c r="F5">
+        <v>175.45</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <f t="shared" si="0"/>
+        <v>2028</v>
+      </c>
+      <c r="B6" t="s">
+        <v>49</v>
+      </c>
+      <c r="C6">
+        <v>409.73</v>
+      </c>
+      <c r="D6">
+        <v>342.66</v>
+      </c>
+      <c r="E6">
+        <v>355.23</v>
+      </c>
+      <c r="F6">
+        <v>175.45</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <f t="shared" si="0"/>
+        <v>2029</v>
+      </c>
+      <c r="B7" t="s">
+        <v>49</v>
+      </c>
+      <c r="C7">
+        <v>409.73</v>
+      </c>
+      <c r="D7">
+        <v>342.66</v>
+      </c>
+      <c r="E7">
+        <v>355.23</v>
+      </c>
+      <c r="F7">
+        <v>175.45</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <f t="shared" si="0"/>
+        <v>2030</v>
+      </c>
+      <c r="B8" t="s">
+        <v>49</v>
+      </c>
+      <c r="C8">
+        <v>409.73</v>
+      </c>
+      <c r="D8">
+        <v>342.66</v>
+      </c>
+      <c r="E8">
+        <v>355.23</v>
+      </c>
+      <c r="F8">
+        <v>175.45</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A9">
+        <f t="shared" si="0"/>
+        <v>2031</v>
+      </c>
+      <c r="B9" t="s">
+        <v>49</v>
+      </c>
+      <c r="C9">
+        <v>409.73</v>
+      </c>
+      <c r="D9">
+        <v>342.66</v>
+      </c>
+      <c r="E9">
+        <v>355.23</v>
+      </c>
+      <c r="F9">
+        <v>175.45</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A10">
+        <f t="shared" si="0"/>
+        <v>2032</v>
+      </c>
+      <c r="B10" t="s">
+        <v>49</v>
+      </c>
+      <c r="C10">
+        <v>409.73</v>
+      </c>
+      <c r="D10">
+        <v>342.66</v>
+      </c>
+      <c r="E10">
+        <v>355.23</v>
+      </c>
+      <c r="F10">
+        <v>175.45</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A11">
+        <f t="shared" si="0"/>
+        <v>2033</v>
+      </c>
+      <c r="B11" t="s">
+        <v>49</v>
+      </c>
+      <c r="C11">
+        <v>409.73</v>
+      </c>
+      <c r="D11">
+        <v>342.66</v>
+      </c>
+      <c r="E11">
+        <v>355.23</v>
+      </c>
+      <c r="F11">
+        <v>175.45</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A12">
+        <f t="shared" si="0"/>
+        <v>2034</v>
+      </c>
+      <c r="B12" t="s">
+        <v>49</v>
+      </c>
+      <c r="C12">
+        <v>409.73</v>
+      </c>
+      <c r="D12">
+        <v>342.66</v>
+      </c>
+      <c r="E12">
+        <v>355.23</v>
+      </c>
+      <c r="F12">
+        <v>175.45</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A13">
+        <f t="shared" si="0"/>
+        <v>2035</v>
+      </c>
+      <c r="B13" t="s">
+        <v>49</v>
+      </c>
+      <c r="C13">
+        <v>409.73</v>
+      </c>
+      <c r="D13">
+        <v>342.66</v>
+      </c>
+      <c r="E13">
+        <v>355.23</v>
+      </c>
+      <c r="F13">
+        <v>175.45</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A14">
+        <f t="shared" si="0"/>
+        <v>2036</v>
+      </c>
+      <c r="B14" t="s">
+        <v>49</v>
+      </c>
+      <c r="C14">
+        <v>409.73</v>
+      </c>
+      <c r="D14">
+        <v>342.66</v>
+      </c>
+      <c r="E14">
+        <v>355.23</v>
+      </c>
+      <c r="F14">
+        <v>175.45</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A15">
+        <f t="shared" si="0"/>
+        <v>2037</v>
+      </c>
+      <c r="B15" t="s">
+        <v>49</v>
+      </c>
+      <c r="C15">
+        <v>409.73</v>
+      </c>
+      <c r="D15">
+        <v>342.66</v>
+      </c>
+      <c r="E15">
+        <v>355.23</v>
+      </c>
+      <c r="F15">
+        <v>175.45</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A16">
+        <f t="shared" si="0"/>
+        <v>2038</v>
+      </c>
+      <c r="B16" t="s">
+        <v>49</v>
+      </c>
+      <c r="C16">
+        <v>409.73</v>
+      </c>
+      <c r="D16">
+        <v>342.66</v>
+      </c>
+      <c r="E16">
+        <v>355.23</v>
+      </c>
+      <c r="F16">
+        <v>175.45</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A17">
+        <f t="shared" si="0"/>
+        <v>2039</v>
+      </c>
+      <c r="B17" t="s">
+        <v>49</v>
+      </c>
+      <c r="C17">
+        <v>409.73</v>
+      </c>
+      <c r="D17">
+        <v>342.66</v>
+      </c>
+      <c r="E17">
+        <v>355.23</v>
+      </c>
+      <c r="F17">
+        <v>175.45</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A18">
+        <f t="shared" si="0"/>
+        <v>2040</v>
+      </c>
+      <c r="B18" t="s">
+        <v>49</v>
+      </c>
+      <c r="C18">
+        <v>409.73</v>
+      </c>
+      <c r="D18">
+        <v>342.66</v>
+      </c>
+      <c r="E18">
+        <v>355.23</v>
+      </c>
+      <c r="F18">
+        <v>175.45</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A19">
+        <f t="shared" si="0"/>
+        <v>2041</v>
+      </c>
+      <c r="B19" t="s">
+        <v>49</v>
+      </c>
+      <c r="C19">
+        <v>409.73</v>
+      </c>
+      <c r="D19">
+        <v>342.66</v>
+      </c>
+      <c r="E19">
+        <v>355.23</v>
+      </c>
+      <c r="F19">
+        <v>175.45</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A20">
+        <f t="shared" si="0"/>
+        <v>2042</v>
+      </c>
+      <c r="B20" t="s">
+        <v>49</v>
+      </c>
+      <c r="C20">
+        <v>409.73</v>
+      </c>
+      <c r="D20">
+        <v>342.66</v>
+      </c>
+      <c r="E20">
+        <v>355.23</v>
+      </c>
+      <c r="F20">
+        <v>175.45</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A21">
+        <f t="shared" si="0"/>
+        <v>2043</v>
+      </c>
+      <c r="B21" t="s">
+        <v>49</v>
+      </c>
+      <c r="C21">
+        <v>409.73</v>
+      </c>
+      <c r="D21">
+        <v>342.66</v>
+      </c>
+      <c r="E21">
+        <v>355.23</v>
+      </c>
+      <c r="F21">
+        <v>175.45</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A22">
+        <f t="shared" si="0"/>
+        <v>2044</v>
+      </c>
+      <c r="B22" t="s">
+        <v>49</v>
+      </c>
+      <c r="C22">
+        <v>409.73</v>
+      </c>
+      <c r="D22">
+        <v>342.66</v>
+      </c>
+      <c r="E22">
+        <v>355.23</v>
+      </c>
+      <c r="F22">
+        <v>175.45</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A23">
+        <f t="shared" si="0"/>
+        <v>2045</v>
+      </c>
+      <c r="B23" t="s">
+        <v>49</v>
+      </c>
+      <c r="C23">
+        <v>409.73</v>
+      </c>
+      <c r="D23">
+        <v>342.66</v>
+      </c>
+      <c r="E23">
+        <v>355.23</v>
+      </c>
+      <c r="F23">
+        <v>175.45</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A24">
+        <f t="shared" si="0"/>
+        <v>2046</v>
+      </c>
+      <c r="B24" t="s">
+        <v>49</v>
+      </c>
+      <c r="C24">
+        <v>409.73</v>
+      </c>
+      <c r="D24">
+        <v>342.66</v>
+      </c>
+      <c r="E24">
+        <v>355.23</v>
+      </c>
+      <c r="F24">
+        <v>175.45</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A25">
+        <f t="shared" si="0"/>
+        <v>2047</v>
+      </c>
+      <c r="B25" t="s">
+        <v>49</v>
+      </c>
+      <c r="C25">
+        <v>409.73</v>
+      </c>
+      <c r="D25">
+        <v>342.66</v>
+      </c>
+      <c r="E25">
+        <v>355.23</v>
+      </c>
+      <c r="F25">
+        <v>175.45</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A26">
+        <f t="shared" si="0"/>
+        <v>2048</v>
+      </c>
+      <c r="B26" t="s">
+        <v>49</v>
+      </c>
+      <c r="C26">
+        <v>409.73</v>
+      </c>
+      <c r="D26">
+        <v>342.66</v>
+      </c>
+      <c r="E26">
+        <v>355.23</v>
+      </c>
+      <c r="F26">
+        <v>175.45</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A27">
+        <f t="shared" si="0"/>
+        <v>2049</v>
+      </c>
+      <c r="B27" t="s">
+        <v>49</v>
+      </c>
+      <c r="C27">
+        <v>409.73</v>
+      </c>
+      <c r="D27">
+        <v>342.66</v>
+      </c>
+      <c r="E27">
+        <v>355.23</v>
+      </c>
+      <c r="F27">
+        <v>175.45</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A28">
+        <f t="shared" si="0"/>
+        <v>2050</v>
+      </c>
+      <c r="B28" t="s">
+        <v>49</v>
+      </c>
+      <c r="C28">
+        <v>409.73</v>
+      </c>
+      <c r="D28">
+        <v>342.66</v>
+      </c>
+      <c r="E28">
+        <v>355.23</v>
+      </c>
+      <c r="F28">
+        <v>175.45</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A29">
+        <f t="shared" si="0"/>
+        <v>2051</v>
+      </c>
+      <c r="B29" t="s">
+        <v>49</v>
+      </c>
+      <c r="C29">
+        <v>409.73</v>
+      </c>
+      <c r="D29">
+        <v>342.66</v>
+      </c>
+      <c r="E29">
+        <v>355.23</v>
+      </c>
+      <c r="F29">
+        <v>175.45</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A30">
+        <f t="shared" si="0"/>
+        <v>2052</v>
+      </c>
+      <c r="B30" t="s">
+        <v>49</v>
+      </c>
+      <c r="C30">
+        <v>409.73</v>
+      </c>
+      <c r="D30">
+        <v>342.66</v>
+      </c>
+      <c r="E30">
+        <v>355.23</v>
+      </c>
+      <c r="F30">
+        <v>175.45</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A31">
+        <f t="shared" si="0"/>
+        <v>2053</v>
+      </c>
+      <c r="B31" t="s">
+        <v>49</v>
+      </c>
+      <c r="C31">
+        <v>409.73</v>
+      </c>
+      <c r="D31">
+        <v>342.66</v>
+      </c>
+      <c r="E31">
+        <v>355.23</v>
+      </c>
+      <c r="F31">
+        <v>175.45</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A32">
+        <f t="shared" si="0"/>
+        <v>2054</v>
+      </c>
+      <c r="B32" t="s">
+        <v>49</v>
+      </c>
+      <c r="C32">
+        <v>409.73</v>
+      </c>
+      <c r="D32">
+        <v>342.66</v>
+      </c>
+      <c r="E32">
+        <v>355.23</v>
+      </c>
+      <c r="F32">
+        <v>175.45</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A33">
+        <f t="shared" si="0"/>
+        <v>2055</v>
+      </c>
+      <c r="B33" t="s">
+        <v>49</v>
+      </c>
+      <c r="C33">
+        <v>409.73</v>
+      </c>
+      <c r="D33">
+        <v>342.66</v>
+      </c>
+      <c r="E33">
+        <v>355.23</v>
+      </c>
+      <c r="F33">
+        <v>175.45</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A34">
+        <f t="shared" si="0"/>
+        <v>2056</v>
+      </c>
+      <c r="B34" t="s">
+        <v>49</v>
+      </c>
+      <c r="C34">
+        <v>409.73</v>
+      </c>
+      <c r="D34">
+        <v>342.66</v>
+      </c>
+      <c r="E34">
+        <v>355.23</v>
+      </c>
+      <c r="F34">
+        <v>175.45</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A35">
+        <f t="shared" si="0"/>
+        <v>2057</v>
+      </c>
+      <c r="B35" t="s">
+        <v>49</v>
+      </c>
+      <c r="C35">
+        <v>409.73</v>
+      </c>
+      <c r="D35">
+        <v>342.66</v>
+      </c>
+      <c r="E35">
+        <v>355.23</v>
+      </c>
+      <c r="F35">
+        <v>175.45</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A36">
+        <f t="shared" si="0"/>
+        <v>2058</v>
+      </c>
+      <c r="B36" t="s">
+        <v>49</v>
+      </c>
+      <c r="C36">
+        <v>409.73</v>
+      </c>
+      <c r="D36">
+        <v>342.66</v>
+      </c>
+      <c r="E36">
+        <v>355.23</v>
+      </c>
+      <c r="F36">
+        <v>175.45</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A37">
+        <f t="shared" si="0"/>
+        <v>2059</v>
+      </c>
+      <c r="B37" t="s">
+        <v>49</v>
+      </c>
+      <c r="C37">
+        <v>409.73</v>
+      </c>
+      <c r="D37">
+        <v>342.66</v>
+      </c>
+      <c r="E37">
+        <v>355.23</v>
+      </c>
+      <c r="F37">
+        <v>175.45</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A38">
+        <f t="shared" si="0"/>
+        <v>2060</v>
+      </c>
+      <c r="B38" t="s">
+        <v>49</v>
+      </c>
+      <c r="C38">
+        <v>409.73</v>
+      </c>
+      <c r="D38">
+        <v>342.66</v>
+      </c>
+      <c r="E38">
+        <v>355.23</v>
+      </c>
+      <c r="F38">
+        <v>175.45</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A39">
+        <f t="shared" si="0"/>
+        <v>2061</v>
+      </c>
+      <c r="B39" t="s">
+        <v>49</v>
+      </c>
+      <c r="C39">
+        <v>409.73</v>
+      </c>
+      <c r="D39">
+        <v>342.66</v>
+      </c>
+      <c r="E39">
+        <v>355.23</v>
+      </c>
+      <c r="F39">
+        <v>175.45</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A40">
+        <f t="shared" si="0"/>
+        <v>2062</v>
+      </c>
+      <c r="B40" t="s">
+        <v>49</v>
+      </c>
+      <c r="C40">
+        <v>409.73</v>
+      </c>
+      <c r="D40">
+        <v>342.66</v>
+      </c>
+      <c r="E40">
+        <v>355.23</v>
+      </c>
+      <c r="F40">
+        <v>175.45</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A41">
+        <f t="shared" si="0"/>
+        <v>2063</v>
+      </c>
+      <c r="B41" t="s">
+        <v>49</v>
+      </c>
+      <c r="C41">
+        <v>409.73</v>
+      </c>
+      <c r="D41">
+        <v>342.66</v>
+      </c>
+      <c r="E41">
+        <v>355.23</v>
+      </c>
+      <c r="F41">
+        <v>175.45</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A42">
+        <f t="shared" si="0"/>
+        <v>2064</v>
+      </c>
+      <c r="B42" t="s">
+        <v>49</v>
+      </c>
+      <c r="C42">
+        <v>409.73</v>
+      </c>
+      <c r="D42">
+        <v>342.66</v>
+      </c>
+      <c r="E42">
+        <v>355.23</v>
+      </c>
+      <c r="F42">
+        <v>175.45</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A43">
+        <f t="shared" si="0"/>
+        <v>2065</v>
+      </c>
+      <c r="B43" t="s">
+        <v>49</v>
+      </c>
+      <c r="C43">
+        <v>409.73</v>
+      </c>
+      <c r="D43">
+        <v>342.66</v>
+      </c>
+      <c r="E43">
+        <v>355.23</v>
+      </c>
+      <c r="F43">
+        <v>175.45</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A44">
+        <f t="shared" si="0"/>
+        <v>2066</v>
+      </c>
+      <c r="B44" t="s">
+        <v>49</v>
+      </c>
+      <c r="C44">
+        <v>409.73</v>
+      </c>
+      <c r="D44">
+        <v>342.66</v>
+      </c>
+      <c r="E44">
+        <v>355.23</v>
+      </c>
+      <c r="F44">
+        <v>175.45</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A45">
+        <f t="shared" si="0"/>
+        <v>2067</v>
+      </c>
+      <c r="B45" t="s">
+        <v>49</v>
+      </c>
+      <c r="C45">
+        <v>409.73</v>
+      </c>
+      <c r="D45">
+        <v>342.66</v>
+      </c>
+      <c r="E45">
+        <v>355.23</v>
+      </c>
+      <c r="F45">
+        <v>175.45</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A46">
+        <f t="shared" si="0"/>
+        <v>2068</v>
+      </c>
+      <c r="B46" t="s">
+        <v>49</v>
+      </c>
+      <c r="C46">
+        <v>409.73</v>
+      </c>
+      <c r="D46">
+        <v>342.66</v>
+      </c>
+      <c r="E46">
+        <v>355.23</v>
+      </c>
+      <c r="F46">
+        <v>175.45</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A47">
+        <f t="shared" si="0"/>
+        <v>2069</v>
+      </c>
+      <c r="B47" t="s">
+        <v>49</v>
+      </c>
+      <c r="C47">
+        <v>409.73</v>
+      </c>
+      <c r="D47">
+        <v>342.66</v>
+      </c>
+      <c r="E47">
+        <v>355.23</v>
+      </c>
+      <c r="F47">
+        <v>175.45</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A48">
+        <f t="shared" si="0"/>
+        <v>2070</v>
+      </c>
+      <c r="B48" t="s">
+        <v>49</v>
+      </c>
+      <c r="C48">
+        <v>409.73</v>
+      </c>
+      <c r="D48">
+        <v>342.66</v>
+      </c>
+      <c r="E48">
+        <v>355.23</v>
+      </c>
+      <c r="F48">
+        <v>175.45</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A49">
+        <f t="shared" si="0"/>
+        <v>2071</v>
+      </c>
+      <c r="B49" t="s">
+        <v>49</v>
+      </c>
+      <c r="C49">
+        <v>409.73</v>
+      </c>
+      <c r="D49">
+        <v>342.66</v>
+      </c>
+      <c r="E49">
+        <v>355.23</v>
+      </c>
+      <c r="F49">
+        <v>175.45</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A50">
+        <f t="shared" si="0"/>
+        <v>2072</v>
+      </c>
+      <c r="B50" t="s">
+        <v>49</v>
+      </c>
+      <c r="C50">
+        <v>409.73</v>
+      </c>
+      <c r="D50">
+        <v>342.66</v>
+      </c>
+      <c r="E50">
+        <v>355.23</v>
+      </c>
+      <c r="F50">
+        <v>175.45</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A51">
+        <f t="shared" si="0"/>
+        <v>2073</v>
+      </c>
+      <c r="B51" t="s">
+        <v>49</v>
+      </c>
+      <c r="C51">
+        <v>409.73</v>
+      </c>
+      <c r="D51">
+        <v>342.66</v>
+      </c>
+      <c r="E51">
+        <v>355.23</v>
+      </c>
+      <c r="F51">
+        <v>175.45</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A52">
+        <f t="shared" si="0"/>
+        <v>2074</v>
+      </c>
+      <c r="B52" t="s">
+        <v>49</v>
+      </c>
+      <c r="C52">
+        <v>409.73</v>
+      </c>
+      <c r="D52">
+        <v>342.66</v>
+      </c>
+      <c r="E52">
+        <v>355.23</v>
+      </c>
+      <c r="F52">
+        <v>175.45</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A53">
+        <f t="shared" si="0"/>
+        <v>2075</v>
+      </c>
+      <c r="B53" t="s">
+        <v>49</v>
+      </c>
+      <c r="C53">
+        <v>409.73</v>
+      </c>
+      <c r="D53">
+        <v>342.66</v>
+      </c>
+      <c r="E53">
+        <v>355.23</v>
+      </c>
+      <c r="F53">
+        <v>175.45</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A54">
+        <f t="shared" si="0"/>
+        <v>2076</v>
+      </c>
+      <c r="B54" t="s">
+        <v>49</v>
+      </c>
+      <c r="C54">
+        <v>409.73</v>
+      </c>
+      <c r="D54">
+        <v>342.66</v>
+      </c>
+      <c r="E54">
+        <v>355.23</v>
+      </c>
+      <c r="F54">
+        <v>175.45</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A55">
+        <f t="shared" si="0"/>
+        <v>2077</v>
+      </c>
+      <c r="B55" t="s">
+        <v>49</v>
+      </c>
+      <c r="C55">
+        <v>409.73</v>
+      </c>
+      <c r="D55">
+        <v>342.66</v>
+      </c>
+      <c r="E55">
+        <v>355.23</v>
+      </c>
+      <c r="F55">
+        <v>175.45</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A56">
+        <f t="shared" si="0"/>
+        <v>2078</v>
+      </c>
+      <c r="B56" t="s">
+        <v>49</v>
+      </c>
+      <c r="C56">
+        <v>409.73</v>
+      </c>
+      <c r="D56">
+        <v>342.66</v>
+      </c>
+      <c r="E56">
+        <v>355.23</v>
+      </c>
+      <c r="F56">
+        <v>175.45</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A57">
+        <f t="shared" si="0"/>
+        <v>2079</v>
+      </c>
+      <c r="B57" t="s">
+        <v>49</v>
+      </c>
+      <c r="C57">
+        <v>409.73</v>
+      </c>
+      <c r="D57">
+        <v>342.66</v>
+      </c>
+      <c r="E57">
+        <v>355.23</v>
+      </c>
+      <c r="F57">
+        <v>175.45</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A58">
+        <f t="shared" si="0"/>
+        <v>2080</v>
+      </c>
+      <c r="B58" t="s">
+        <v>49</v>
+      </c>
+      <c r="C58">
+        <v>409.73</v>
+      </c>
+      <c r="D58">
+        <v>342.66</v>
+      </c>
+      <c r="E58">
+        <v>355.23</v>
+      </c>
+      <c r="F58">
         <v>175.45</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Added mock fleet proportion dataset
</commit_message>
<xml_diff>
--- a/data/MetCouncilTables.xlsx
+++ b/data/MetCouncilTables.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://icfonline-my.sharepoint.com/personal/61886_icf_com/Documents/Desktop/transport-emission-shiny/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="25" documentId="8_{BBC49CD7-68E0-4D8F-B576-EE14E509F0DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9A42A5A0-4EEB-4C5D-A128-675A4F344D14}"/>
+  <xr:revisionPtr revIDLastSave="52" documentId="8_{BBC49CD7-68E0-4D8F-B576-EE14E509F0DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{235B5D1A-0A6F-4A49-A773-A53767DBAF2D}"/>
   <bookViews>
-    <workbookView minimized="1" xWindow="345" yWindow="675" windowWidth="27645" windowHeight="15150" firstSheet="1" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView minimized="1" xWindow="840" yWindow="735" windowWidth="18225" windowHeight="15150" firstSheet="17" activeTab="19" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ProjectTypes" sheetId="1" r:id="rId1"/>
@@ -32,6 +32,7 @@
     <sheet name="ImpactOfCapacityExpansion " sheetId="32" r:id="rId17"/>
     <sheet name="TotalLifecycleGHGs" sheetId="39" r:id="rId18"/>
     <sheet name="SocialCostCarbon" sheetId="40" r:id="rId19"/>
+    <sheet name="FleetProportion" sheetId="41" r:id="rId20"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -51,7 +52,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="507" uniqueCount="200">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="512" uniqueCount="200">
   <si>
     <t>category</t>
   </si>
@@ -701,7 +702,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -710,6 +711,7 @@
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -5384,6 +5386,1076 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AC17391B-F9D1-4FA3-B95E-4F95F46E1D6D}">
+  <dimension ref="A1:E62"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="14" customWidth="1"/>
+    <col min="3" max="3" width="22.7109375" customWidth="1"/>
+    <col min="4" max="4" width="21.7109375" customWidth="1"/>
+    <col min="5" max="5" width="25.42578125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1" s="6" t="s">
+        <v>199</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>2020</v>
+      </c>
+      <c r="B2">
+        <v>90</v>
+      </c>
+      <c r="C2">
+        <v>4</v>
+      </c>
+      <c r="D2">
+        <v>0.01</v>
+      </c>
+      <c r="E2">
+        <v>5.99</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>2021</v>
+      </c>
+      <c r="B3">
+        <v>90</v>
+      </c>
+      <c r="C3">
+        <v>4</v>
+      </c>
+      <c r="D3">
+        <v>0.01</v>
+      </c>
+      <c r="E3">
+        <v>5.99</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>2022</v>
+      </c>
+      <c r="B4">
+        <v>90</v>
+      </c>
+      <c r="C4">
+        <v>4</v>
+      </c>
+      <c r="D4">
+        <v>0.01</v>
+      </c>
+      <c r="E4">
+        <v>5.99</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>2023</v>
+      </c>
+      <c r="B5">
+        <v>90</v>
+      </c>
+      <c r="C5">
+        <v>4</v>
+      </c>
+      <c r="D5">
+        <v>0.01</v>
+      </c>
+      <c r="E5">
+        <v>5.99</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>2024</v>
+      </c>
+      <c r="B6">
+        <v>90</v>
+      </c>
+      <c r="C6">
+        <v>4</v>
+      </c>
+      <c r="D6">
+        <v>0.01</v>
+      </c>
+      <c r="E6">
+        <v>5.99</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>2025</v>
+      </c>
+      <c r="B7">
+        <v>90</v>
+      </c>
+      <c r="C7">
+        <v>4</v>
+      </c>
+      <c r="D7">
+        <v>0.01</v>
+      </c>
+      <c r="E7">
+        <v>5.99</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <v>2026</v>
+      </c>
+      <c r="B8">
+        <v>90</v>
+      </c>
+      <c r="C8">
+        <v>4</v>
+      </c>
+      <c r="D8">
+        <v>0.01</v>
+      </c>
+      <c r="E8">
+        <v>5.99</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A9">
+        <v>2027</v>
+      </c>
+      <c r="B9">
+        <v>90</v>
+      </c>
+      <c r="C9">
+        <v>4</v>
+      </c>
+      <c r="D9">
+        <v>0.01</v>
+      </c>
+      <c r="E9">
+        <v>5.99</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A10">
+        <v>2028</v>
+      </c>
+      <c r="B10">
+        <v>90</v>
+      </c>
+      <c r="C10">
+        <v>4</v>
+      </c>
+      <c r="D10">
+        <v>0.01</v>
+      </c>
+      <c r="E10">
+        <v>5.99</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A11">
+        <v>2029</v>
+      </c>
+      <c r="B11">
+        <v>90</v>
+      </c>
+      <c r="C11">
+        <v>4</v>
+      </c>
+      <c r="D11">
+        <v>0.01</v>
+      </c>
+      <c r="E11">
+        <v>5.99</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A12">
+        <v>2030</v>
+      </c>
+      <c r="B12">
+        <v>90</v>
+      </c>
+      <c r="C12">
+        <v>4</v>
+      </c>
+      <c r="D12">
+        <v>0.01</v>
+      </c>
+      <c r="E12">
+        <v>5.99</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A13">
+        <v>2031</v>
+      </c>
+      <c r="B13">
+        <v>90</v>
+      </c>
+      <c r="C13">
+        <v>4</v>
+      </c>
+      <c r="D13">
+        <v>0.01</v>
+      </c>
+      <c r="E13">
+        <v>5.99</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A14">
+        <v>2032</v>
+      </c>
+      <c r="B14">
+        <v>90</v>
+      </c>
+      <c r="C14">
+        <v>4</v>
+      </c>
+      <c r="D14">
+        <v>0.01</v>
+      </c>
+      <c r="E14">
+        <v>5.99</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A15">
+        <v>2033</v>
+      </c>
+      <c r="B15">
+        <v>90</v>
+      </c>
+      <c r="C15">
+        <v>4</v>
+      </c>
+      <c r="D15">
+        <v>0.01</v>
+      </c>
+      <c r="E15">
+        <v>5.99</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A16">
+        <v>2034</v>
+      </c>
+      <c r="B16">
+        <v>90</v>
+      </c>
+      <c r="C16">
+        <v>4</v>
+      </c>
+      <c r="D16">
+        <v>0.01</v>
+      </c>
+      <c r="E16">
+        <v>5.99</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A17">
+        <v>2035</v>
+      </c>
+      <c r="B17">
+        <v>90</v>
+      </c>
+      <c r="C17">
+        <v>4</v>
+      </c>
+      <c r="D17">
+        <v>0.01</v>
+      </c>
+      <c r="E17">
+        <v>5.99</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A18">
+        <v>2036</v>
+      </c>
+      <c r="B18">
+        <v>90</v>
+      </c>
+      <c r="C18">
+        <v>4</v>
+      </c>
+      <c r="D18">
+        <v>0.01</v>
+      </c>
+      <c r="E18">
+        <v>5.99</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A19">
+        <v>2037</v>
+      </c>
+      <c r="B19">
+        <v>90</v>
+      </c>
+      <c r="C19">
+        <v>4</v>
+      </c>
+      <c r="D19">
+        <v>0.01</v>
+      </c>
+      <c r="E19">
+        <v>5.99</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A20">
+        <v>2038</v>
+      </c>
+      <c r="B20">
+        <v>90</v>
+      </c>
+      <c r="C20">
+        <v>4</v>
+      </c>
+      <c r="D20">
+        <v>0.01</v>
+      </c>
+      <c r="E20">
+        <v>5.99</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A21">
+        <v>2039</v>
+      </c>
+      <c r="B21">
+        <v>90</v>
+      </c>
+      <c r="C21">
+        <v>4</v>
+      </c>
+      <c r="D21">
+        <v>0.01</v>
+      </c>
+      <c r="E21">
+        <v>5.99</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A22">
+        <v>2040</v>
+      </c>
+      <c r="B22">
+        <v>90</v>
+      </c>
+      <c r="C22">
+        <v>4</v>
+      </c>
+      <c r="D22">
+        <v>0.01</v>
+      </c>
+      <c r="E22">
+        <v>5.99</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A23">
+        <v>2041</v>
+      </c>
+      <c r="B23">
+        <v>90</v>
+      </c>
+      <c r="C23">
+        <v>4</v>
+      </c>
+      <c r="D23">
+        <v>0.01</v>
+      </c>
+      <c r="E23">
+        <v>5.99</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A24">
+        <v>2042</v>
+      </c>
+      <c r="B24">
+        <v>90</v>
+      </c>
+      <c r="C24">
+        <v>4</v>
+      </c>
+      <c r="D24">
+        <v>0.01</v>
+      </c>
+      <c r="E24">
+        <v>5.99</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A25">
+        <v>2043</v>
+      </c>
+      <c r="B25">
+        <v>90</v>
+      </c>
+      <c r="C25">
+        <v>4</v>
+      </c>
+      <c r="D25">
+        <v>0.01</v>
+      </c>
+      <c r="E25">
+        <v>5.99</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A26">
+        <v>2044</v>
+      </c>
+      <c r="B26">
+        <v>90</v>
+      </c>
+      <c r="C26">
+        <v>4</v>
+      </c>
+      <c r="D26">
+        <v>0.01</v>
+      </c>
+      <c r="E26">
+        <v>5.99</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A27">
+        <v>2045</v>
+      </c>
+      <c r="B27">
+        <v>90</v>
+      </c>
+      <c r="C27">
+        <v>4</v>
+      </c>
+      <c r="D27">
+        <v>0.01</v>
+      </c>
+      <c r="E27">
+        <v>5.99</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A28">
+        <v>2046</v>
+      </c>
+      <c r="B28">
+        <v>90</v>
+      </c>
+      <c r="C28">
+        <v>4</v>
+      </c>
+      <c r="D28">
+        <v>0.01</v>
+      </c>
+      <c r="E28">
+        <v>5.99</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A29">
+        <v>2047</v>
+      </c>
+      <c r="B29">
+        <v>90</v>
+      </c>
+      <c r="C29">
+        <v>4</v>
+      </c>
+      <c r="D29">
+        <v>0.01</v>
+      </c>
+      <c r="E29">
+        <v>5.99</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A30">
+        <v>2048</v>
+      </c>
+      <c r="B30">
+        <v>90</v>
+      </c>
+      <c r="C30">
+        <v>4</v>
+      </c>
+      <c r="D30">
+        <v>0.01</v>
+      </c>
+      <c r="E30">
+        <v>5.99</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A31">
+        <v>2049</v>
+      </c>
+      <c r="B31">
+        <v>90</v>
+      </c>
+      <c r="C31">
+        <v>4</v>
+      </c>
+      <c r="D31">
+        <v>0.01</v>
+      </c>
+      <c r="E31">
+        <v>5.99</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A32">
+        <v>2050</v>
+      </c>
+      <c r="B32">
+        <v>90</v>
+      </c>
+      <c r="C32">
+        <v>4</v>
+      </c>
+      <c r="D32">
+        <v>0.01</v>
+      </c>
+      <c r="E32">
+        <v>5.99</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A33">
+        <v>2051</v>
+      </c>
+      <c r="B33">
+        <v>90</v>
+      </c>
+      <c r="C33">
+        <v>4</v>
+      </c>
+      <c r="D33">
+        <v>0.01</v>
+      </c>
+      <c r="E33">
+        <v>5.99</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A34">
+        <v>2052</v>
+      </c>
+      <c r="B34">
+        <v>90</v>
+      </c>
+      <c r="C34">
+        <v>4</v>
+      </c>
+      <c r="D34">
+        <v>0.01</v>
+      </c>
+      <c r="E34">
+        <v>5.99</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A35">
+        <v>2053</v>
+      </c>
+      <c r="B35">
+        <v>90</v>
+      </c>
+      <c r="C35">
+        <v>4</v>
+      </c>
+      <c r="D35">
+        <v>0.01</v>
+      </c>
+      <c r="E35">
+        <v>5.99</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A36">
+        <v>2054</v>
+      </c>
+      <c r="B36">
+        <v>90</v>
+      </c>
+      <c r="C36">
+        <v>4</v>
+      </c>
+      <c r="D36">
+        <v>0.01</v>
+      </c>
+      <c r="E36">
+        <v>5.99</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A37">
+        <v>2055</v>
+      </c>
+      <c r="B37">
+        <v>90</v>
+      </c>
+      <c r="C37">
+        <v>4</v>
+      </c>
+      <c r="D37">
+        <v>0.01</v>
+      </c>
+      <c r="E37">
+        <v>5.99</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A38">
+        <v>2056</v>
+      </c>
+      <c r="B38">
+        <v>90</v>
+      </c>
+      <c r="C38">
+        <v>4</v>
+      </c>
+      <c r="D38">
+        <v>0.01</v>
+      </c>
+      <c r="E38">
+        <v>5.99</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A39">
+        <v>2057</v>
+      </c>
+      <c r="B39">
+        <v>90</v>
+      </c>
+      <c r="C39">
+        <v>4</v>
+      </c>
+      <c r="D39">
+        <v>0.01</v>
+      </c>
+      <c r="E39">
+        <v>5.99</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A40">
+        <v>2058</v>
+      </c>
+      <c r="B40">
+        <v>90</v>
+      </c>
+      <c r="C40">
+        <v>4</v>
+      </c>
+      <c r="D40">
+        <v>0.01</v>
+      </c>
+      <c r="E40">
+        <v>5.99</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A41">
+        <v>2059</v>
+      </c>
+      <c r="B41">
+        <v>90</v>
+      </c>
+      <c r="C41">
+        <v>4</v>
+      </c>
+      <c r="D41">
+        <v>0.01</v>
+      </c>
+      <c r="E41">
+        <v>5.99</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A42">
+        <v>2060</v>
+      </c>
+      <c r="B42">
+        <v>90</v>
+      </c>
+      <c r="C42">
+        <v>4</v>
+      </c>
+      <c r="D42">
+        <v>0.01</v>
+      </c>
+      <c r="E42">
+        <v>5.99</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A43">
+        <v>2061</v>
+      </c>
+      <c r="B43">
+        <v>90</v>
+      </c>
+      <c r="C43">
+        <v>4</v>
+      </c>
+      <c r="D43">
+        <v>0.01</v>
+      </c>
+      <c r="E43">
+        <v>5.99</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A44">
+        <v>2062</v>
+      </c>
+      <c r="B44">
+        <v>90</v>
+      </c>
+      <c r="C44">
+        <v>4</v>
+      </c>
+      <c r="D44">
+        <v>0.01</v>
+      </c>
+      <c r="E44">
+        <v>5.99</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A45">
+        <v>2063</v>
+      </c>
+      <c r="B45">
+        <v>90</v>
+      </c>
+      <c r="C45">
+        <v>4</v>
+      </c>
+      <c r="D45">
+        <v>0.01</v>
+      </c>
+      <c r="E45">
+        <v>5.99</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A46">
+        <v>2064</v>
+      </c>
+      <c r="B46">
+        <v>90</v>
+      </c>
+      <c r="C46">
+        <v>4</v>
+      </c>
+      <c r="D46">
+        <v>0.01</v>
+      </c>
+      <c r="E46">
+        <v>5.99</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A47">
+        <v>2065</v>
+      </c>
+      <c r="B47">
+        <v>90</v>
+      </c>
+      <c r="C47">
+        <v>4</v>
+      </c>
+      <c r="D47">
+        <v>0.01</v>
+      </c>
+      <c r="E47">
+        <v>5.99</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A48">
+        <v>2066</v>
+      </c>
+      <c r="B48">
+        <v>90</v>
+      </c>
+      <c r="C48">
+        <v>4</v>
+      </c>
+      <c r="D48">
+        <v>0.01</v>
+      </c>
+      <c r="E48">
+        <v>5.99</v>
+      </c>
+    </row>
+    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A49">
+        <v>2067</v>
+      </c>
+      <c r="B49">
+        <v>90</v>
+      </c>
+      <c r="C49">
+        <v>4</v>
+      </c>
+      <c r="D49">
+        <v>0.01</v>
+      </c>
+      <c r="E49">
+        <v>5.99</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A50">
+        <v>2068</v>
+      </c>
+      <c r="B50">
+        <v>90</v>
+      </c>
+      <c r="C50">
+        <v>4</v>
+      </c>
+      <c r="D50">
+        <v>0.01</v>
+      </c>
+      <c r="E50">
+        <v>5.99</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A51">
+        <v>2069</v>
+      </c>
+      <c r="B51">
+        <v>90</v>
+      </c>
+      <c r="C51">
+        <v>4</v>
+      </c>
+      <c r="D51">
+        <v>0.01</v>
+      </c>
+      <c r="E51">
+        <v>5.99</v>
+      </c>
+    </row>
+    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A52">
+        <v>2070</v>
+      </c>
+      <c r="B52">
+        <v>90</v>
+      </c>
+      <c r="C52">
+        <v>4</v>
+      </c>
+      <c r="D52">
+        <v>0.01</v>
+      </c>
+      <c r="E52">
+        <v>5.99</v>
+      </c>
+    </row>
+    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A53">
+        <v>2071</v>
+      </c>
+      <c r="B53">
+        <v>90</v>
+      </c>
+      <c r="C53">
+        <v>4</v>
+      </c>
+      <c r="D53">
+        <v>0.01</v>
+      </c>
+      <c r="E53">
+        <v>5.99</v>
+      </c>
+    </row>
+    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A54">
+        <v>2072</v>
+      </c>
+      <c r="B54">
+        <v>90</v>
+      </c>
+      <c r="C54">
+        <v>4</v>
+      </c>
+      <c r="D54">
+        <v>0.01</v>
+      </c>
+      <c r="E54">
+        <v>5.99</v>
+      </c>
+    </row>
+    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A55">
+        <v>2073</v>
+      </c>
+      <c r="B55">
+        <v>90</v>
+      </c>
+      <c r="C55">
+        <v>4</v>
+      </c>
+      <c r="D55">
+        <v>0.01</v>
+      </c>
+      <c r="E55">
+        <v>5.99</v>
+      </c>
+    </row>
+    <row r="56" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A56">
+        <v>2074</v>
+      </c>
+      <c r="B56">
+        <v>90</v>
+      </c>
+      <c r="C56">
+        <v>4</v>
+      </c>
+      <c r="D56">
+        <v>0.01</v>
+      </c>
+      <c r="E56">
+        <v>5.99</v>
+      </c>
+    </row>
+    <row r="57" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A57">
+        <v>2075</v>
+      </c>
+      <c r="B57">
+        <v>90</v>
+      </c>
+      <c r="C57">
+        <v>4</v>
+      </c>
+      <c r="D57">
+        <v>0.01</v>
+      </c>
+      <c r="E57">
+        <v>5.99</v>
+      </c>
+    </row>
+    <row r="58" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A58">
+        <v>2076</v>
+      </c>
+      <c r="B58">
+        <v>90</v>
+      </c>
+      <c r="C58">
+        <v>4</v>
+      </c>
+      <c r="D58">
+        <v>0.01</v>
+      </c>
+      <c r="E58">
+        <v>5.99</v>
+      </c>
+    </row>
+    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A59">
+        <v>2077</v>
+      </c>
+      <c r="B59">
+        <v>90</v>
+      </c>
+      <c r="C59">
+        <v>4</v>
+      </c>
+      <c r="D59">
+        <v>0.01</v>
+      </c>
+      <c r="E59">
+        <v>5.99</v>
+      </c>
+    </row>
+    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A60">
+        <v>2078</v>
+      </c>
+      <c r="B60">
+        <v>90</v>
+      </c>
+      <c r="C60">
+        <v>4</v>
+      </c>
+      <c r="D60">
+        <v>0.01</v>
+      </c>
+      <c r="E60">
+        <v>5.99</v>
+      </c>
+    </row>
+    <row r="61" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A61">
+        <v>2079</v>
+      </c>
+      <c r="B61">
+        <v>90</v>
+      </c>
+      <c r="C61">
+        <v>4</v>
+      </c>
+      <c r="D61">
+        <v>0.01</v>
+      </c>
+      <c r="E61">
+        <v>5.99</v>
+      </c>
+    </row>
+    <row r="62" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A62">
+        <v>2080</v>
+      </c>
+      <c r="B62">
+        <v>90</v>
+      </c>
+      <c r="C62">
+        <v>4</v>
+      </c>
+      <c r="D62">
+        <v>0.01</v>
+      </c>
+      <c r="E62">
+        <v>5.99</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:C8"/>
@@ -6995,6 +8067,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
   <dimension ref="A1:C8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="30.85546875" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">

</xml_diff>

<commit_message>
electrification outreach first go
</commit_message>
<xml_diff>
--- a/data/MetCouncilTables.xlsx
+++ b/data/MetCouncilTables.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="27531"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="27726"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://icfonline-my.sharepoint.com/personal/61886_icf_com/Documents/Desktop/transport-emission-shiny/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="52" documentId="8_{BBC49CD7-68E0-4D8F-B576-EE14E509F0DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{235B5D1A-0A6F-4A49-A773-A53767DBAF2D}"/>
+  <xr:revisionPtr revIDLastSave="56" documentId="8_{BBC49CD7-68E0-4D8F-B576-EE14E509F0DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{10826B05-2296-4509-A3DA-91B5E18C4EF1}"/>
   <bookViews>
-    <workbookView minimized="1" xWindow="840" yWindow="735" windowWidth="18225" windowHeight="15150" firstSheet="17" activeTab="19" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-30" yWindow="0" windowWidth="14385" windowHeight="15450" firstSheet="7" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ProjectTypes" sheetId="1" r:id="rId1"/>
@@ -8069,6 +8069,8 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="30.85546875" customWidth="1"/>
+    <col min="2" max="2" width="27.28515625" customWidth="1"/>
+    <col min="3" max="3" width="24.5703125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.25">
@@ -8168,6 +8170,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0B00-000000000000}">
   <dimension ref="A1:B7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="35.140625" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:2" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">

</xml_diff>

<commit_message>
Added trip distance data
</commit_message>
<xml_diff>
--- a/data/MetCouncilTables.xlsx
+++ b/data/MetCouncilTables.xlsx
@@ -8,31 +8,32 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://icfonline-my.sharepoint.com/personal/61886_icf_com/Documents/Desktop/transport-emission-shiny/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="109" documentId="8_{BBC49CD7-68E0-4D8F-B576-EE14E509F0DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5ADC5D89-2176-4841-82AA-74B7EDC1E369}"/>
+  <xr:revisionPtr revIDLastSave="111" documentId="8_{BBC49CD7-68E0-4D8F-B576-EE14E509F0DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A8A4BF36-BB07-4B76-8C7B-C7002FFAE4C1}"/>
   <bookViews>
-    <workbookView xWindow="13950" yWindow="0" windowWidth="14745" windowHeight="15450" firstSheet="13" activeTab="13" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="ProjectTypes" sheetId="1" r:id="rId1"/>
-    <sheet name="DefaultLifetime" sheetId="2" r:id="rId2"/>
-    <sheet name="TransitDependencyAdjustments" sheetId="4" r:id="rId3"/>
-    <sheet name="GREETCarbonIntensity" sheetId="5" r:id="rId4"/>
-    <sheet name="MobilityServiceVMTReduction" sheetId="6" r:id="rId5"/>
-    <sheet name="OCTAMobilityHubVMT" sheetId="7" r:id="rId6"/>
-    <sheet name="AccesstoTransitImpact" sheetId="8" r:id="rId7"/>
-    <sheet name="AdjustmentFactorsAndTripLengths" sheetId="11" r:id="rId8"/>
-    <sheet name="TotalVMTReductionPotential" sheetId="12" r:id="rId9"/>
-    <sheet name="ElasticityOfRidershipIncrease" sheetId="14" r:id="rId10"/>
-    <sheet name="RecommendedBRTImpactAssumptions" sheetId="15" r:id="rId11"/>
-    <sheet name="TripAndVMTModeShiftPotential" sheetId="19" r:id="rId12"/>
-    <sheet name="EnergyEfficiencyForEVs" sheetId="20" r:id="rId13"/>
-    <sheet name="ModeShiftFactor" sheetId="22" r:id="rId14"/>
-    <sheet name="CreditForKeyDestinations" sheetId="23" r:id="rId15"/>
-    <sheet name="FuelConsumptionAtIdle" sheetId="28" r:id="rId16"/>
-    <sheet name="ImpactOfCapacityExpansion " sheetId="32" r:id="rId17"/>
-    <sheet name="TotalLifecycleGHGs" sheetId="39" r:id="rId18"/>
-    <sheet name="SocialCostCarbon" sheetId="40" r:id="rId19"/>
-    <sheet name="FleetProportion" sheetId="41" r:id="rId20"/>
+    <sheet name="TripDistances" sheetId="42" r:id="rId1"/>
+    <sheet name="ProjectTypes" sheetId="1" r:id="rId2"/>
+    <sheet name="DefaultLifetime" sheetId="2" r:id="rId3"/>
+    <sheet name="TransitDependencyAdjustments" sheetId="4" r:id="rId4"/>
+    <sheet name="GREETCarbonIntensity" sheetId="5" r:id="rId5"/>
+    <sheet name="MobilityServiceVMTReduction" sheetId="6" r:id="rId6"/>
+    <sheet name="OCTAMobilityHubVMT" sheetId="7" r:id="rId7"/>
+    <sheet name="AccesstoTransitImpact" sheetId="8" r:id="rId8"/>
+    <sheet name="AdjustmentFactorsAndTripLengths" sheetId="11" r:id="rId9"/>
+    <sheet name="TotalVMTReductionPotential" sheetId="12" r:id="rId10"/>
+    <sheet name="ElasticityOfRidershipIncrease" sheetId="14" r:id="rId11"/>
+    <sheet name="RecommendedBRTImpactAssumptions" sheetId="15" r:id="rId12"/>
+    <sheet name="TripAndVMTModeShiftPotential" sheetId="19" r:id="rId13"/>
+    <sheet name="EnergyEfficiencyForEVs" sheetId="20" r:id="rId14"/>
+    <sheet name="ModeShiftFactor" sheetId="22" r:id="rId15"/>
+    <sheet name="CreditForKeyDestinations" sheetId="23" r:id="rId16"/>
+    <sheet name="FuelConsumptionAtIdle" sheetId="28" r:id="rId17"/>
+    <sheet name="ImpactOfCapacityExpansion " sheetId="32" r:id="rId18"/>
+    <sheet name="TotalLifecycleGHGs" sheetId="39" r:id="rId19"/>
+    <sheet name="SocialCostCarbon" sheetId="40" r:id="rId20"/>
+    <sheet name="FleetProportion" sheetId="41" r:id="rId21"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -52,7 +53,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="512" uniqueCount="200">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="537" uniqueCount="223">
   <si>
     <t>category</t>
   </si>
@@ -652,6 +653,75 @@
   </si>
   <si>
     <t>Year</t>
+  </si>
+  <si>
+    <t>mode_type</t>
+  </si>
+  <si>
+    <t>distance_avg</t>
+  </si>
+  <si>
+    <t>distance_avg_low</t>
+  </si>
+  <si>
+    <t>distance_avg_upp</t>
+  </si>
+  <si>
+    <t>distance_median</t>
+  </si>
+  <si>
+    <t>distance_median_low</t>
+  </si>
+  <si>
+    <t>distance_median_upp</t>
+  </si>
+  <si>
+    <t>count</t>
+  </si>
+  <si>
+    <t>Bicycle</t>
+  </si>
+  <si>
+    <t>For-Hire Vehicle</t>
+  </si>
+  <si>
+    <t>NA</t>
+  </si>
+  <si>
+    <t>Household Vehicle</t>
+  </si>
+  <si>
+    <t>Long distance passenger mode</t>
+  </si>
+  <si>
+    <t>Micromobility</t>
+  </si>
+  <si>
+    <t>Missing</t>
+  </si>
+  <si>
+    <t>Other</t>
+  </si>
+  <si>
+    <t>Other Bus</t>
+  </si>
+  <si>
+    <t>Other Vehicle</t>
+  </si>
+  <si>
+    <t>Public Bus</t>
+  </si>
+  <si>
+    <t>Rail</t>
+  </si>
+  <si>
+    <t>School Bus</t>
+  </si>
+  <si>
+    <t>Smartphone ridehailing service</t>
+  </si>
+  <si>
+    <t>Walk</t>
   </si>
 </sst>
 </file>
@@ -1015,100 +1085,398 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B11"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6342DC05-FA87-40E6-A32B-A06CC074627B}">
+  <dimension ref="A1:H15"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="31.140625" customWidth="1"/>
-    <col min="2" max="2" width="46.42578125" customWidth="1"/>
-  </cols>
   <sheetData>
-    <row r="1" spans="1:2" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>200</v>
+      </c>
+      <c r="B1" t="s">
+        <v>201</v>
+      </c>
+      <c r="C1" t="s">
+        <v>202</v>
+      </c>
+      <c r="D1" t="s">
+        <v>203</v>
+      </c>
+      <c r="E1" t="s">
+        <v>204</v>
+      </c>
+      <c r="F1" t="s">
+        <v>205</v>
+      </c>
+      <c r="G1" t="s">
+        <v>206</v>
+      </c>
+      <c r="H1" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>208</v>
+      </c>
+      <c r="B2">
+        <v>2.9749119231916001</v>
+      </c>
+      <c r="C2">
+        <v>2.4119651827793902</v>
+      </c>
+      <c r="D2">
+        <v>3.5378586636037999</v>
+      </c>
+      <c r="E2">
+        <v>1.54680046864397</v>
+      </c>
+      <c r="F2">
+        <v>1.23623681666273</v>
+      </c>
+      <c r="G2">
+        <v>2.0965177550660798</v>
+      </c>
+      <c r="H2">
+        <v>537</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>209</v>
+      </c>
+      <c r="B3">
+        <v>3.6999170502861798</v>
+      </c>
+      <c r="C3">
+        <v>2.5538506463772901</v>
+      </c>
+      <c r="D3">
+        <v>4.8459834541950704</v>
+      </c>
+      <c r="E3">
+        <v>4.2547154693920097</v>
+      </c>
+      <c r="F3">
+        <v>4.2547154693920097</v>
+      </c>
+      <c r="G3" t="s">
+        <v>210</v>
+      </c>
+      <c r="H3">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>211</v>
+      </c>
+      <c r="B4">
+        <v>5.9016230035503296</v>
+      </c>
+      <c r="C4">
+        <v>5.7355947620142604</v>
+      </c>
+      <c r="D4">
+        <v>6.0676512450864104</v>
+      </c>
+      <c r="E4">
+        <v>3.6316722396401402</v>
+      </c>
+      <c r="F4">
+        <v>3.5184190209222801</v>
+      </c>
+      <c r="G4">
+        <v>3.7296255253294799</v>
+      </c>
+      <c r="H4">
+        <v>24661</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>212</v>
+      </c>
+      <c r="B5">
+        <v>3.8634645109851302</v>
+      </c>
+      <c r="C5">
+        <v>3.8634645109851302</v>
+      </c>
+      <c r="D5">
+        <v>3.8634645109851302</v>
+      </c>
+      <c r="E5">
+        <v>3.8634645109851302</v>
+      </c>
+      <c r="F5" t="s">
+        <v>210</v>
+      </c>
+      <c r="G5" t="s">
+        <v>210</v>
+      </c>
+      <c r="H5">
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>2</v>
-      </c>
-      <c r="B2" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>2</v>
-      </c>
-      <c r="B3" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>5</v>
-      </c>
-      <c r="B4" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>5</v>
-      </c>
-      <c r="B5" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
+        <v>213</v>
+      </c>
+      <c r="B6">
+        <v>0.71198948216291502</v>
+      </c>
+      <c r="C6">
+        <v>0.389736805991869</v>
+      </c>
+      <c r="D6">
+        <v>1.03424215833396</v>
+      </c>
+      <c r="E6">
+        <v>0.50182283165373298</v>
+      </c>
+      <c r="F6">
+        <v>0.34792776009053</v>
+      </c>
+      <c r="G6">
+        <v>1.48653150978066</v>
+      </c>
+      <c r="H6">
         <v>8</v>
       </c>
-      <c r="B6" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>8</v>
-      </c>
-      <c r="B7" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+        <v>214</v>
+      </c>
+      <c r="B7">
+        <v>0.97570910188785598</v>
+      </c>
+      <c r="C7">
+        <v>0.678877459679468</v>
+      </c>
+      <c r="D7">
+        <v>1.27254074409624</v>
+      </c>
+      <c r="E7">
+        <v>0.30579813491132901</v>
+      </c>
+      <c r="F7">
+        <v>0.26405217382669199</v>
+      </c>
+      <c r="G7">
+        <v>0.38299261169806598</v>
+      </c>
+      <c r="H7">
+        <v>744</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>11</v>
-      </c>
-      <c r="B8" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+        <v>215</v>
+      </c>
+      <c r="B8">
+        <v>6.4778152091502204</v>
+      </c>
+      <c r="C8">
+        <v>3.9201240751621702</v>
+      </c>
+      <c r="D8">
+        <v>9.0355063431382696</v>
+      </c>
+      <c r="E8">
+        <v>3.1503708159140298</v>
+      </c>
+      <c r="F8">
+        <v>1.98401869924806</v>
+      </c>
+      <c r="G8">
+        <v>5.0317932725823402</v>
+      </c>
+      <c r="H8">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>11</v>
-      </c>
-      <c r="B9" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+        <v>216</v>
+      </c>
+      <c r="B9">
+        <v>7.7004599845074297</v>
+      </c>
+      <c r="C9">
+        <v>0.19012344959704799</v>
+      </c>
+      <c r="D9">
+        <v>15.2107965194178</v>
+      </c>
+      <c r="E9">
+        <v>3.5798176526679</v>
+      </c>
+      <c r="F9">
+        <v>2.1826241499209398</v>
+      </c>
+      <c r="G9">
+        <v>5.53153176776941</v>
+      </c>
+      <c r="H9">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>14</v>
-      </c>
-      <c r="B10" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+        <v>217</v>
+      </c>
+      <c r="B10">
+        <v>5.8322002863550404</v>
+      </c>
+      <c r="C10">
+        <v>5.2493400278704199</v>
+      </c>
+      <c r="D10">
+        <v>6.4150605448396503</v>
+      </c>
+      <c r="E10">
+        <v>3.4341547328826598</v>
+      </c>
+      <c r="F10">
+        <v>2.84192477033208</v>
+      </c>
+      <c r="G10">
+        <v>3.8088495422747601</v>
+      </c>
+      <c r="H10">
+        <v>1699</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>14</v>
-      </c>
-      <c r="B11" t="s">
-        <v>16</v>
+        <v>218</v>
+      </c>
+      <c r="B11">
+        <v>5.2559515730838502</v>
+      </c>
+      <c r="C11">
+        <v>4.3340884063229499</v>
+      </c>
+      <c r="D11">
+        <v>6.1778147398447603</v>
+      </c>
+      <c r="E11">
+        <v>3.90877999838896</v>
+      </c>
+      <c r="F11">
+        <v>2.5543898528153401</v>
+      </c>
+      <c r="G11">
+        <v>4.75539530008502</v>
+      </c>
+      <c r="H11">
+        <v>648</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>219</v>
+      </c>
+      <c r="B12">
+        <v>4.3043541561638703</v>
+      </c>
+      <c r="C12">
+        <v>3.5978914187361402</v>
+      </c>
+      <c r="D12">
+        <v>5.0108168935915902</v>
+      </c>
+      <c r="E12">
+        <v>3.4614622327978899</v>
+      </c>
+      <c r="F12">
+        <v>2.7029974008196498</v>
+      </c>
+      <c r="G12">
+        <v>5.7456170381036502</v>
+      </c>
+      <c r="H12">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>220</v>
+      </c>
+      <c r="B13">
+        <v>4.4554427783066402</v>
+      </c>
+      <c r="C13">
+        <v>2.9360163676167201</v>
+      </c>
+      <c r="D13">
+        <v>5.9748691889965704</v>
+      </c>
+      <c r="E13">
+        <v>2.05524454125531</v>
+      </c>
+      <c r="F13">
+        <v>1.8132993857604001</v>
+      </c>
+      <c r="G13">
+        <v>2.6033558726978798</v>
+      </c>
+      <c r="H13">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>221</v>
+      </c>
+      <c r="B14">
+        <v>5.8745743082736501</v>
+      </c>
+      <c r="C14">
+        <v>4.7868159756589401</v>
+      </c>
+      <c r="D14">
+        <v>6.9623326408883504</v>
+      </c>
+      <c r="E14">
+        <v>5.6432568002624199</v>
+      </c>
+      <c r="F14">
+        <v>2.5407774758494401</v>
+      </c>
+      <c r="G14">
+        <v>6.4024709173268803</v>
+      </c>
+      <c r="H14">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>222</v>
+      </c>
+      <c r="B15">
+        <v>0.85801128591603704</v>
+      </c>
+      <c r="C15">
+        <v>0.69649622674294198</v>
+      </c>
+      <c r="D15">
+        <v>1.0195263450891301</v>
+      </c>
+      <c r="E15">
+        <v>0.368423768732074</v>
+      </c>
+      <c r="F15">
+        <v>0.34324348797476201</v>
+      </c>
+      <c r="G15">
+        <v>0.39342064566496898</v>
+      </c>
+      <c r="H15">
+        <v>4415</v>
       </c>
     </row>
   </sheetData>
@@ -1117,6 +1485,75 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0B00-000000000000}">
+  <dimension ref="A1:B7"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="35.140625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>54</v>
+      </c>
+      <c r="B2" s="3">
+        <v>5.8000000000000003E-2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>55</v>
+      </c>
+      <c r="B3" s="3">
+        <v>2.64E-2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>56</v>
+      </c>
+      <c r="B4" s="3">
+        <v>2.6700000000000002E-2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>57</v>
+      </c>
+      <c r="B5" s="3">
+        <v>4.8000000000000001E-2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>58</v>
+      </c>
+      <c r="B6" s="3">
+        <v>5.3100000000000001E-2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>59</v>
+      </c>
+      <c r="B7" s="3">
+        <v>9.4500000000000001E-2</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0D00-000000000000}">
   <dimension ref="A1:F3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1177,7 +1614,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0E00-000000000000}">
   <dimension ref="A1:D5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1257,7 +1694,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1200-000000000000}">
   <dimension ref="A1:E3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1318,7 +1755,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1300-000000000000}">
   <dimension ref="A1:C6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1399,7 +1836,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1500-000000000000}">
   <dimension ref="A1:D10"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1540,7 +1977,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1600-000000000000}">
   <dimension ref="A1:C5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1605,7 +2042,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1B00-000000000000}">
   <dimension ref="A1:E12"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1798,7 +2235,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1F00-000000000000}">
   <dimension ref="A1:E13"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2032,7 +2469,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-2600-000000000000}">
   <dimension ref="A1:E7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2155,7 +2592,109 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:B11"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="31.140625" customWidth="1"/>
+    <col min="2" max="2" width="46.42578125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>5</v>
+      </c>
+      <c r="B4" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>5</v>
+      </c>
+      <c r="B5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>8</v>
+      </c>
+      <c r="B6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>8</v>
+      </c>
+      <c r="B7" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>11</v>
+      </c>
+      <c r="B8" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>11</v>
+      </c>
+      <c r="B9" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>14</v>
+      </c>
+      <c r="B10" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>14</v>
+      </c>
+      <c r="B11" t="s">
+        <v>16</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FC06F369-1B95-458E-A555-6CC2EF2B1D77}">
   <dimension ref="A1:E184"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -5293,105 +5832,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:C8"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData>
-    <row r="1" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B2">
-        <v>4</v>
-      </c>
-      <c r="C2" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>22</v>
-      </c>
-      <c r="B3">
-        <v>5</v>
-      </c>
-      <c r="C3" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>24</v>
-      </c>
-      <c r="B4">
-        <v>7</v>
-      </c>
-      <c r="C4" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>26</v>
-      </c>
-      <c r="B5">
-        <v>8</v>
-      </c>
-      <c r="C5" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>28</v>
-      </c>
-      <c r="B6">
-        <v>10</v>
-      </c>
-      <c r="C6" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>30</v>
-      </c>
-      <c r="B7">
-        <v>14</v>
-      </c>
-      <c r="C7" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>32</v>
-      </c>
-      <c r="B8">
-        <v>20</v>
-      </c>
-      <c r="C8" t="s">
-        <v>33</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AC17391B-F9D1-4FA3-B95E-4F95F46E1D6D}">
   <dimension ref="A1:E62"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -6462,6 +6903,104 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <dimension ref="A1:C8"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B2">
+        <v>4</v>
+      </c>
+      <c r="C2" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>22</v>
+      </c>
+      <c r="B3">
+        <v>5</v>
+      </c>
+      <c r="C3" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>24</v>
+      </c>
+      <c r="B4">
+        <v>7</v>
+      </c>
+      <c r="C4" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>26</v>
+      </c>
+      <c r="B5">
+        <v>8</v>
+      </c>
+      <c r="C5" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>28</v>
+      </c>
+      <c r="B6">
+        <v>10</v>
+      </c>
+      <c r="C6" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>30</v>
+      </c>
+      <c r="B7">
+        <v>14</v>
+      </c>
+      <c r="C7" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>32</v>
+      </c>
+      <c r="B8">
+        <v>20</v>
+      </c>
+      <c r="C8" t="s">
+        <v>33</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:C8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -6559,7 +7098,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:G58"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -7789,7 +8328,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:D8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -7911,7 +8450,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:D5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -7991,7 +8530,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <dimension ref="A1:D6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -8068,7 +8607,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
   <dimension ref="A1:C8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -8169,73 +8708,4 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0B00-000000000000}">
-  <dimension ref="A1:B7"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="35.140625" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:2" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>78</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>54</v>
-      </c>
-      <c r="B2" s="3">
-        <v>5.8000000000000003E-2</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>55</v>
-      </c>
-      <c r="B3" s="3">
-        <v>2.64E-2</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>56</v>
-      </c>
-      <c r="B4" s="3">
-        <v>2.6700000000000002E-2</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>57</v>
-      </c>
-      <c r="B5" s="3">
-        <v>4.8000000000000001E-2</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>58</v>
-      </c>
-      <c r="B6" s="3">
-        <v>5.3100000000000001E-2</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>59</v>
-      </c>
-      <c r="B7" s="3">
-        <v>9.4500000000000001E-2</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
adding daily vmt by community type
</commit_message>
<xml_diff>
--- a/data/MetCouncilTables.xlsx
+++ b/data/MetCouncilTables.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="27726"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27726"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://icfonline-my.sharepoint.com/personal/61886_icf_com/Documents/Desktop/transport-emission-shiny/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="111" documentId="8_{BBC49CD7-68E0-4D8F-B576-EE14E509F0DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A8A4BF36-BB07-4B76-8C7B-C7002FFAE4C1}"/>
+  <xr:revisionPtr revIDLastSave="117" documentId="8_{BBC49CD7-68E0-4D8F-B576-EE14E509F0DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F87D0107-E08D-476B-984C-FE1C7AA834D2}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="8" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="TripDistances" sheetId="42" r:id="rId1"/>
@@ -22,18 +22,19 @@
     <sheet name="OCTAMobilityHubVMT" sheetId="7" r:id="rId7"/>
     <sheet name="AccesstoTransitImpact" sheetId="8" r:id="rId8"/>
     <sheet name="AdjustmentFactorsAndTripLengths" sheetId="11" r:id="rId9"/>
-    <sheet name="TotalVMTReductionPotential" sheetId="12" r:id="rId10"/>
-    <sheet name="ElasticityOfRidershipIncrease" sheetId="14" r:id="rId11"/>
-    <sheet name="RecommendedBRTImpactAssumptions" sheetId="15" r:id="rId12"/>
-    <sheet name="TripAndVMTModeShiftPotential" sheetId="19" r:id="rId13"/>
-    <sheet name="EnergyEfficiencyForEVs" sheetId="20" r:id="rId14"/>
-    <sheet name="ModeShiftFactor" sheetId="22" r:id="rId15"/>
-    <sheet name="CreditForKeyDestinations" sheetId="23" r:id="rId16"/>
-    <sheet name="FuelConsumptionAtIdle" sheetId="28" r:id="rId17"/>
-    <sheet name="ImpactOfCapacityExpansion " sheetId="32" r:id="rId18"/>
-    <sheet name="TotalLifecycleGHGs" sheetId="39" r:id="rId19"/>
-    <sheet name="SocialCostCarbon" sheetId="40" r:id="rId20"/>
-    <sheet name="FleetProportion" sheetId="41" r:id="rId21"/>
+    <sheet name="VMTByCommunityType" sheetId="44" r:id="rId10"/>
+    <sheet name="TotalVMTReductionPotential" sheetId="12" r:id="rId11"/>
+    <sheet name="ElasticityOfRidershipIncrease" sheetId="14" r:id="rId12"/>
+    <sheet name="RecommendedBRTImpactAssumptions" sheetId="15" r:id="rId13"/>
+    <sheet name="TripAndVMTModeShiftPotential" sheetId="19" r:id="rId14"/>
+    <sheet name="EnergyEfficiencyForEVs" sheetId="20" r:id="rId15"/>
+    <sheet name="ModeShiftFactor" sheetId="22" r:id="rId16"/>
+    <sheet name="CreditForKeyDestinations" sheetId="23" r:id="rId17"/>
+    <sheet name="FuelConsumptionAtIdle" sheetId="28" r:id="rId18"/>
+    <sheet name="ImpactOfCapacityExpansion " sheetId="32" r:id="rId19"/>
+    <sheet name="TotalLifecycleGHGs" sheetId="39" r:id="rId20"/>
+    <sheet name="SocialCostCarbon" sheetId="40" r:id="rId21"/>
+    <sheet name="FleetProportion" sheetId="41" r:id="rId22"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -53,7 +54,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="537" uniqueCount="223">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="561" uniqueCount="236">
   <si>
     <t>category</t>
   </si>
@@ -722,13 +723,52 @@
   </si>
   <si>
     <t>Walk</t>
+  </si>
+  <si>
+    <t>survey_year</t>
+  </si>
+  <si>
+    <t>vmt_mid</t>
+  </si>
+  <si>
+    <t>vmt_mid_low</t>
+  </si>
+  <si>
+    <t>vmt_mid_upp</t>
+  </si>
+  <si>
+    <t>vmt</t>
+  </si>
+  <si>
+    <t>vmt_low</t>
+  </si>
+  <si>
+    <t>vmt_upp</t>
+  </si>
+  <si>
+    <t>cd_year</t>
+  </si>
+  <si>
+    <t>CD</t>
+  </si>
+  <si>
+    <t>Urban</t>
+  </si>
+  <si>
+    <t>Suburban</t>
+  </si>
+  <si>
+    <t>Suburban Edge</t>
+  </si>
+  <si>
+    <t>Rural / Non-Council</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="19" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -751,16 +791,308 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="18"/>
+      <color theme="3"/>
+      <name val="Cambria"/>
+      <family val="2"/>
+      <scheme val="major"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="15"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="13"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF006100"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C0006"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C5700"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF3F3F76"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF3F3F3F"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FF7F7F7F"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="33">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA5A5A5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.79998168889431442"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.59999389629810485"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.39997558519241921"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.79998168889431442"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.59999389629810485"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.39997558519241921"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.79998168889431442"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.59999389629810485"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.39997558519241921"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.79998168889431442"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.59999389629810485"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.39997558519241921"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.79998168889431442"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.59999389629810485"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.39997558519241921"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.79998168889431442"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.59999389629810485"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.39997558519241921"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -768,11 +1100,159 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thick">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thick">
+        <color theme="4" tint="0.499984740745262"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4" tint="0.39997558519241921"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF7F7F7F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF7F7F7F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF7F7F7F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF7F7F7F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="double">
+        <color rgb="FFFF8001"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="double">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="double">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="double">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="double">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFB2B2B2"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFB2B2B2"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFB2B2B2"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFB2B2B2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4"/>
+      </top>
+      <bottom style="double">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="13" fillId="6" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="15" fillId="7" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="8" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="18" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="18" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="18" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="18" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="18" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="18" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -782,9 +1262,51 @@
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="42">
+    <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
+    <cellStyle name="20% - Accent2" xfId="23" builtinId="34" customBuiltin="1"/>
+    <cellStyle name="20% - Accent3" xfId="27" builtinId="38" customBuiltin="1"/>
+    <cellStyle name="20% - Accent4" xfId="31" builtinId="42" customBuiltin="1"/>
+    <cellStyle name="20% - Accent5" xfId="35" builtinId="46" customBuiltin="1"/>
+    <cellStyle name="20% - Accent6" xfId="39" builtinId="50" customBuiltin="1"/>
+    <cellStyle name="40% - Accent1" xfId="20" builtinId="31" customBuiltin="1"/>
+    <cellStyle name="40% - Accent2" xfId="24" builtinId="35" customBuiltin="1"/>
+    <cellStyle name="40% - Accent3" xfId="28" builtinId="39" customBuiltin="1"/>
+    <cellStyle name="40% - Accent4" xfId="32" builtinId="43" customBuiltin="1"/>
+    <cellStyle name="40% - Accent5" xfId="36" builtinId="47" customBuiltin="1"/>
+    <cellStyle name="40% - Accent6" xfId="40" builtinId="51" customBuiltin="1"/>
+    <cellStyle name="60% - Accent1" xfId="21" builtinId="32" customBuiltin="1"/>
+    <cellStyle name="60% - Accent2" xfId="25" builtinId="36" customBuiltin="1"/>
+    <cellStyle name="60% - Accent3" xfId="29" builtinId="40" customBuiltin="1"/>
+    <cellStyle name="60% - Accent4" xfId="33" builtinId="44" customBuiltin="1"/>
+    <cellStyle name="60% - Accent5" xfId="37" builtinId="48" customBuiltin="1"/>
+    <cellStyle name="60% - Accent6" xfId="41" builtinId="52" customBuiltin="1"/>
+    <cellStyle name="Accent1" xfId="18" builtinId="29" customBuiltin="1"/>
+    <cellStyle name="Accent2" xfId="22" builtinId="33" customBuiltin="1"/>
+    <cellStyle name="Accent3" xfId="26" builtinId="37" customBuiltin="1"/>
+    <cellStyle name="Accent4" xfId="30" builtinId="41" customBuiltin="1"/>
+    <cellStyle name="Accent5" xfId="34" builtinId="45" customBuiltin="1"/>
+    <cellStyle name="Accent6" xfId="38" builtinId="49" customBuiltin="1"/>
+    <cellStyle name="Bad" xfId="7" builtinId="27" customBuiltin="1"/>
+    <cellStyle name="Calculation" xfId="11" builtinId="22" customBuiltin="1"/>
+    <cellStyle name="Check Cell" xfId="13" builtinId="23" customBuiltin="1"/>
+    <cellStyle name="Explanatory Text" xfId="16" builtinId="53" customBuiltin="1"/>
+    <cellStyle name="Good" xfId="6" builtinId="26" customBuiltin="1"/>
+    <cellStyle name="Heading 1" xfId="2" builtinId="16" customBuiltin="1"/>
+    <cellStyle name="Heading 2" xfId="3" builtinId="17" customBuiltin="1"/>
+    <cellStyle name="Heading 3" xfId="4" builtinId="18" customBuiltin="1"/>
+    <cellStyle name="Heading 4" xfId="5" builtinId="19" customBuiltin="1"/>
+    <cellStyle name="Input" xfId="9" builtinId="20" customBuiltin="1"/>
+    <cellStyle name="Linked Cell" xfId="12" builtinId="24" customBuiltin="1"/>
+    <cellStyle name="Neutral" xfId="8" builtinId="28" customBuiltin="1"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Note" xfId="15" builtinId="10" customBuiltin="1"/>
+    <cellStyle name="Output" xfId="10" builtinId="21" customBuiltin="1"/>
+    <cellStyle name="Title" xfId="1" builtinId="15" customBuiltin="1"/>
+    <cellStyle name="Total" xfId="17" builtinId="25" customBuiltin="1"/>
+    <cellStyle name="Warning Text" xfId="14" builtinId="11" customBuiltin="1"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
@@ -1485,6 +2007,496 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{78DDE928-5E41-4857-9D51-91BD8EEB412E}">
+  <dimension ref="A1:J15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A1" s="7" t="s">
+        <v>223</v>
+      </c>
+      <c r="B1" s="7" t="s">
+        <v>224</v>
+      </c>
+      <c r="C1" s="7" t="s">
+        <v>225</v>
+      </c>
+      <c r="D1" s="7" t="s">
+        <v>226</v>
+      </c>
+      <c r="E1" s="7" t="s">
+        <v>227</v>
+      </c>
+      <c r="F1" s="7" t="s">
+        <v>228</v>
+      </c>
+      <c r="G1" s="7" t="s">
+        <v>229</v>
+      </c>
+      <c r="H1" s="7" t="s">
+        <v>207</v>
+      </c>
+      <c r="I1" s="7" t="s">
+        <v>230</v>
+      </c>
+      <c r="J1" s="7" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A2" s="7">
+        <v>2019</v>
+      </c>
+      <c r="B2" s="7">
+        <v>9.1</v>
+      </c>
+      <c r="C2" s="7">
+        <v>8.4</v>
+      </c>
+      <c r="D2" s="7">
+        <v>9.6</v>
+      </c>
+      <c r="E2" s="7">
+        <v>17.2</v>
+      </c>
+      <c r="F2" s="7">
+        <v>16</v>
+      </c>
+      <c r="G2" s="7">
+        <v>18.3</v>
+      </c>
+      <c r="H2" s="7">
+        <v>11913</v>
+      </c>
+      <c r="I2" s="7">
+        <v>2040</v>
+      </c>
+      <c r="J2" s="7" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A3" s="7">
+        <v>2021</v>
+      </c>
+      <c r="B3" s="7">
+        <v>7.2</v>
+      </c>
+      <c r="C3" s="7">
+        <v>6.7</v>
+      </c>
+      <c r="D3" s="7">
+        <v>7.9</v>
+      </c>
+      <c r="E3" s="7">
+        <v>18.2</v>
+      </c>
+      <c r="F3" s="7">
+        <v>15.4</v>
+      </c>
+      <c r="G3" s="7">
+        <v>21</v>
+      </c>
+      <c r="H3" s="7">
+        <v>9247</v>
+      </c>
+      <c r="I3" s="7">
+        <v>2040</v>
+      </c>
+      <c r="J3" s="7" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A4" s="7">
+        <v>2019</v>
+      </c>
+      <c r="B4" s="7">
+        <v>15.1</v>
+      </c>
+      <c r="C4" s="7">
+        <v>14.4</v>
+      </c>
+      <c r="D4" s="7">
+        <v>16.2</v>
+      </c>
+      <c r="E4" s="7">
+        <v>24.2</v>
+      </c>
+      <c r="F4" s="7">
+        <v>22.8</v>
+      </c>
+      <c r="G4" s="7">
+        <v>25.6</v>
+      </c>
+      <c r="H4" s="7">
+        <v>8366</v>
+      </c>
+      <c r="I4" s="7">
+        <v>2040</v>
+      </c>
+      <c r="J4" s="7" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A5" s="7">
+        <v>2019</v>
+      </c>
+      <c r="B5" s="7">
+        <v>16.600000000000001</v>
+      </c>
+      <c r="C5" s="7">
+        <v>14.3</v>
+      </c>
+      <c r="D5" s="7">
+        <v>18.600000000000001</v>
+      </c>
+      <c r="E5" s="7">
+        <v>25.4</v>
+      </c>
+      <c r="F5" s="7">
+        <v>23.5</v>
+      </c>
+      <c r="G5" s="7">
+        <v>27.2</v>
+      </c>
+      <c r="H5" s="7">
+        <v>1847</v>
+      </c>
+      <c r="I5" s="7">
+        <v>2040</v>
+      </c>
+      <c r="J5" s="7" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A6" s="7">
+        <v>2021</v>
+      </c>
+      <c r="B6" s="7">
+        <v>11.4</v>
+      </c>
+      <c r="C6" s="7">
+        <v>10.199999999999999</v>
+      </c>
+      <c r="D6" s="7">
+        <v>12.5</v>
+      </c>
+      <c r="E6" s="7">
+        <v>27.3</v>
+      </c>
+      <c r="F6" s="7">
+        <v>19.7</v>
+      </c>
+      <c r="G6" s="7">
+        <v>34.9</v>
+      </c>
+      <c r="H6" s="7">
+        <v>4162</v>
+      </c>
+      <c r="I6" s="7">
+        <v>2040</v>
+      </c>
+      <c r="J6" s="7" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A7" s="7">
+        <v>2021</v>
+      </c>
+      <c r="B7" s="7">
+        <v>15</v>
+      </c>
+      <c r="C7" s="7">
+        <v>11.3</v>
+      </c>
+      <c r="D7" s="7">
+        <v>20</v>
+      </c>
+      <c r="E7" s="7">
+        <v>30.7</v>
+      </c>
+      <c r="F7" s="7">
+        <v>23.3</v>
+      </c>
+      <c r="G7" s="7">
+        <v>38.1</v>
+      </c>
+      <c r="H7" s="7">
+        <v>697</v>
+      </c>
+      <c r="I7" s="7">
+        <v>2040</v>
+      </c>
+      <c r="J7" s="7" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A8" s="7">
+        <v>2019</v>
+      </c>
+      <c r="B8" s="7">
+        <v>19.2</v>
+      </c>
+      <c r="C8" s="7">
+        <v>17.600000000000001</v>
+      </c>
+      <c r="D8" s="7">
+        <v>20.7</v>
+      </c>
+      <c r="E8" s="7">
+        <v>32.5</v>
+      </c>
+      <c r="F8" s="7">
+        <v>31</v>
+      </c>
+      <c r="G8" s="7">
+        <v>34</v>
+      </c>
+      <c r="H8" s="7">
+        <v>5952</v>
+      </c>
+      <c r="I8" s="7">
+        <v>2040</v>
+      </c>
+      <c r="J8" s="7" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A9" s="7">
+        <v>2021</v>
+      </c>
+      <c r="B9" s="7">
+        <v>21.2</v>
+      </c>
+      <c r="C9" s="7">
+        <v>17.399999999999999</v>
+      </c>
+      <c r="D9" s="7">
+        <v>24.1</v>
+      </c>
+      <c r="E9" s="7">
+        <v>37.700000000000003</v>
+      </c>
+      <c r="F9" s="7">
+        <v>33.4</v>
+      </c>
+      <c r="G9" s="7">
+        <v>42</v>
+      </c>
+      <c r="H9" s="7">
+        <v>2092</v>
+      </c>
+      <c r="I9" s="7">
+        <v>2040</v>
+      </c>
+      <c r="J9" s="7" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A10" s="7">
+        <v>2019</v>
+      </c>
+      <c r="B10" s="7">
+        <v>9.1999999999999993</v>
+      </c>
+      <c r="C10" s="7">
+        <v>8.6</v>
+      </c>
+      <c r="D10" s="7">
+        <v>9.6999999999999993</v>
+      </c>
+      <c r="E10" s="7">
+        <v>17.399999999999999</v>
+      </c>
+      <c r="F10" s="7">
+        <v>16.3</v>
+      </c>
+      <c r="G10" s="7">
+        <v>18.5</v>
+      </c>
+      <c r="H10" s="7">
+        <v>31037</v>
+      </c>
+      <c r="I10" s="7">
+        <v>2050</v>
+      </c>
+      <c r="J10" s="7" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A11" s="7">
+        <v>2021</v>
+      </c>
+      <c r="B11" s="7">
+        <v>7.2</v>
+      </c>
+      <c r="C11" s="7">
+        <v>6.6</v>
+      </c>
+      <c r="D11" s="7">
+        <v>7.9</v>
+      </c>
+      <c r="E11" s="7">
+        <v>18.100000000000001</v>
+      </c>
+      <c r="F11" s="7">
+        <v>15.5</v>
+      </c>
+      <c r="G11" s="7">
+        <v>20.8</v>
+      </c>
+      <c r="H11" s="7">
+        <v>22131</v>
+      </c>
+      <c r="I11" s="7">
+        <v>2050</v>
+      </c>
+      <c r="J11" s="7" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A12" s="7">
+        <v>2019</v>
+      </c>
+      <c r="B12" s="7">
+        <v>15.4</v>
+      </c>
+      <c r="C12" s="7">
+        <v>14.5</v>
+      </c>
+      <c r="D12" s="7">
+        <v>16.399999999999999</v>
+      </c>
+      <c r="E12" s="7">
+        <v>24.5</v>
+      </c>
+      <c r="F12" s="7">
+        <v>23.2</v>
+      </c>
+      <c r="G12" s="7">
+        <v>25.7</v>
+      </c>
+      <c r="H12" s="7">
+        <v>24506</v>
+      </c>
+      <c r="I12" s="7">
+        <v>2050</v>
+      </c>
+      <c r="J12" s="7" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A13" s="7">
+        <v>2021</v>
+      </c>
+      <c r="B13" s="7">
+        <v>12.2</v>
+      </c>
+      <c r="C13" s="7">
+        <v>11.1</v>
+      </c>
+      <c r="D13" s="7">
+        <v>13.4</v>
+      </c>
+      <c r="E13" s="7">
+        <v>28.4</v>
+      </c>
+      <c r="F13" s="7">
+        <v>21.9</v>
+      </c>
+      <c r="G13" s="7">
+        <v>34.9</v>
+      </c>
+      <c r="H13" s="7">
+        <v>10922</v>
+      </c>
+      <c r="I13" s="7">
+        <v>2050</v>
+      </c>
+      <c r="J13" s="7" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A14" s="7">
+        <v>2019</v>
+      </c>
+      <c r="B14" s="7">
+        <v>19.2</v>
+      </c>
+      <c r="C14" s="7">
+        <v>17.600000000000001</v>
+      </c>
+      <c r="D14" s="7">
+        <v>20.7</v>
+      </c>
+      <c r="E14" s="7">
+        <v>32.5</v>
+      </c>
+      <c r="F14" s="7">
+        <v>31</v>
+      </c>
+      <c r="G14" s="7">
+        <v>34</v>
+      </c>
+      <c r="H14" s="7">
+        <v>14628</v>
+      </c>
+      <c r="I14" s="7">
+        <v>2050</v>
+      </c>
+      <c r="J14" s="7" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A15" s="7">
+        <v>2021</v>
+      </c>
+      <c r="B15" s="7">
+        <v>21.6</v>
+      </c>
+      <c r="C15" s="7">
+        <v>17.5</v>
+      </c>
+      <c r="D15" s="7">
+        <v>24.5</v>
+      </c>
+      <c r="E15" s="7">
+        <v>37.799999999999997</v>
+      </c>
+      <c r="F15" s="7">
+        <v>33.5</v>
+      </c>
+      <c r="G15" s="7">
+        <v>42.1</v>
+      </c>
+      <c r="H15" s="7">
+        <v>4731</v>
+      </c>
+      <c r="I15" s="7">
+        <v>2050</v>
+      </c>
+      <c r="J15" s="7" t="s">
+        <v>235</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0B00-000000000000}">
   <dimension ref="A1:B7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1553,7 +2565,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0D00-000000000000}">
   <dimension ref="A1:F3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1614,7 +2626,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0E00-000000000000}">
   <dimension ref="A1:D5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1694,7 +2706,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1200-000000000000}">
   <dimension ref="A1:E3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1755,7 +2767,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1300-000000000000}">
   <dimension ref="A1:C6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1836,7 +2848,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1500-000000000000}">
   <dimension ref="A1:D10"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1977,7 +2989,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1600-000000000000}">
   <dimension ref="A1:C5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2042,7 +3054,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1B00-000000000000}">
   <dimension ref="A1:E12"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2235,7 +3247,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1F00-000000000000}">
   <dimension ref="A1:E13"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2462,129 +3474,6 @@
       </c>
       <c r="E13" t="s">
         <v>189</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-2600-000000000000}">
-  <dimension ref="A1:E7"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData>
-    <row r="1" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>190</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>167</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>168</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>169</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>171</v>
-      </c>
-      <c r="B2" s="4">
-        <v>6398393</v>
-      </c>
-      <c r="C2" s="4">
-        <v>7886579</v>
-      </c>
-      <c r="D2" s="4">
-        <v>11639444</v>
-      </c>
-      <c r="E2" s="4">
-        <v>11692704</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>172</v>
-      </c>
-      <c r="B3">
-        <v>36.950000000000003</v>
-      </c>
-      <c r="C3">
-        <v>45.55</v>
-      </c>
-      <c r="D3">
-        <v>67.22</v>
-      </c>
-      <c r="E3">
-        <v>67.53</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>173</v>
-      </c>
-      <c r="B4">
-        <v>409.73</v>
-      </c>
-      <c r="C4">
-        <v>409.73</v>
-      </c>
-      <c r="D4">
-        <v>175.45</v>
-      </c>
-      <c r="E4">
-        <v>175.45</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>174</v>
-      </c>
-      <c r="B5" s="3">
-        <v>8.3000000000000004E-2</v>
-      </c>
-      <c r="C5" s="3">
-        <v>0.1</v>
-      </c>
-      <c r="D5" s="3">
-        <v>0.27700000000000002</v>
-      </c>
-      <c r="E5" s="3">
-        <v>0.27800000000000002</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>175</v>
-      </c>
-      <c r="B6">
-        <v>446.68</v>
-      </c>
-      <c r="C6">
-        <v>455.28</v>
-      </c>
-      <c r="D6">
-        <v>242.67</v>
-      </c>
-      <c r="E6">
-        <v>242.98</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>176</v>
-      </c>
-      <c r="D7" s="2">
-        <v>-0.45</v>
-      </c>
-      <c r="E7" s="2">
-        <v>-0.46</v>
       </c>
     </row>
   </sheetData>
@@ -2695,6 +3584,129 @@
 </file>
 
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-2600-000000000000}">
+  <dimension ref="A1:E7"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>190</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>167</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>168</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>169</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>171</v>
+      </c>
+      <c r="B2" s="4">
+        <v>6398393</v>
+      </c>
+      <c r="C2" s="4">
+        <v>7886579</v>
+      </c>
+      <c r="D2" s="4">
+        <v>11639444</v>
+      </c>
+      <c r="E2" s="4">
+        <v>11692704</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>172</v>
+      </c>
+      <c r="B3">
+        <v>36.950000000000003</v>
+      </c>
+      <c r="C3">
+        <v>45.55</v>
+      </c>
+      <c r="D3">
+        <v>67.22</v>
+      </c>
+      <c r="E3">
+        <v>67.53</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>173</v>
+      </c>
+      <c r="B4">
+        <v>409.73</v>
+      </c>
+      <c r="C4">
+        <v>409.73</v>
+      </c>
+      <c r="D4">
+        <v>175.45</v>
+      </c>
+      <c r="E4">
+        <v>175.45</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>174</v>
+      </c>
+      <c r="B5" s="3">
+        <v>8.3000000000000004E-2</v>
+      </c>
+      <c r="C5" s="3">
+        <v>0.1</v>
+      </c>
+      <c r="D5" s="3">
+        <v>0.27700000000000002</v>
+      </c>
+      <c r="E5" s="3">
+        <v>0.27800000000000002</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>175</v>
+      </c>
+      <c r="B6">
+        <v>446.68</v>
+      </c>
+      <c r="C6">
+        <v>455.28</v>
+      </c>
+      <c r="D6">
+        <v>242.67</v>
+      </c>
+      <c r="E6">
+        <v>242.98</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>176</v>
+      </c>
+      <c r="D7" s="2">
+        <v>-0.45</v>
+      </c>
+      <c r="E7" s="2">
+        <v>-0.46</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FC06F369-1B95-458E-A555-6CC2EF2B1D77}">
   <dimension ref="A1:E184"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -5832,7 +6844,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AC17391B-F9D1-4FA3-B95E-4F95F46E1D6D}">
   <dimension ref="A1:E62"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>

</xml_diff>

<commit_message>
writing and adding ev infrastrucutre calculation to server
</commit_message>
<xml_diff>
--- a/data/MetCouncilTables.xlsx
+++ b/data/MetCouncilTables.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://icfonline-my.sharepoint.com/personal/61886_icf_com/Documents/Desktop/transport-emission-shiny/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="154" documentId="8_{BBC49CD7-68E0-4D8F-B576-EE14E509F0DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2CBA9F2C-CDF7-4BE3-BC3C-853E416206BA}"/>
+  <xr:revisionPtr revIDLastSave="167" documentId="8_{BBC49CD7-68E0-4D8F-B576-EE14E509F0DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{55D89571-C465-45CA-8F78-FAE742371238}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="4" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="14310" windowHeight="15480" firstSheet="5" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="TripDistances" sheetId="42" r:id="rId1"/>
@@ -18,24 +18,25 @@
     <sheet name="DefaultLifetime" sheetId="2" r:id="rId3"/>
     <sheet name="TransitDependencyAdjustments" sheetId="4" r:id="rId4"/>
     <sheet name="GREETCarbonIntensity" sheetId="5" r:id="rId5"/>
-    <sheet name="MobilityServiceVMTReduction" sheetId="6" r:id="rId6"/>
-    <sheet name="OCTAMobilityHubVMT" sheetId="7" r:id="rId7"/>
-    <sheet name="AccesstoTransitImpact" sheetId="8" r:id="rId8"/>
-    <sheet name="AdjustmentFactorsAndTripLengths" sheetId="11" r:id="rId9"/>
-    <sheet name="VMTByCommunityType" sheetId="44" r:id="rId10"/>
-    <sheet name="TotalVMTReductionPotential" sheetId="12" r:id="rId11"/>
-    <sheet name="ElasticityOfRidershipIncrease" sheetId="14" r:id="rId12"/>
-    <sheet name="RecommendedBRTImpactAssumptions" sheetId="15" r:id="rId13"/>
-    <sheet name="TripAndVMTModeShiftPotential" sheetId="19" r:id="rId14"/>
-    <sheet name="EnergyEfficiencyForEVs" sheetId="20" r:id="rId15"/>
-    <sheet name="ModeShiftFactor" sheetId="22" r:id="rId16"/>
-    <sheet name="CreditForKeyDestinations" sheetId="23" r:id="rId17"/>
-    <sheet name="FuelConsumptionAtIdle" sheetId="28" r:id="rId18"/>
-    <sheet name="ImpactOfCapacityExpansion " sheetId="32" r:id="rId19"/>
-    <sheet name="TotalLifecycleGHGs" sheetId="39" r:id="rId20"/>
-    <sheet name="SocialCostCarbon" sheetId="40" r:id="rId21"/>
+    <sheet name="FuelEfficiency" sheetId="45" r:id="rId6"/>
+    <sheet name="MobilityServiceVMTReduction" sheetId="6" r:id="rId7"/>
+    <sheet name="OCTAMobilityHubVMT" sheetId="7" r:id="rId8"/>
+    <sheet name="AccesstoTransitImpact" sheetId="8" r:id="rId9"/>
+    <sheet name="AdjustmentFactorsAndTripLengths" sheetId="11" r:id="rId10"/>
+    <sheet name="VMTByCommunityType" sheetId="44" r:id="rId11"/>
+    <sheet name="TotalVMTReductionPotential" sheetId="12" r:id="rId12"/>
+    <sheet name="ElasticityOfRidershipIncrease" sheetId="14" r:id="rId13"/>
+    <sheet name="RecommendedBRTImpactAssumptions" sheetId="15" r:id="rId14"/>
+    <sheet name="TripAndVMTModeShiftPotential" sheetId="19" r:id="rId15"/>
+    <sheet name="EnergyEfficiencyForEVs" sheetId="20" r:id="rId16"/>
+    <sheet name="ModeShiftFactor" sheetId="22" r:id="rId17"/>
+    <sheet name="CreditForKeyDestinations" sheetId="23" r:id="rId18"/>
+    <sheet name="FuelConsumptionAtIdle" sheetId="28" r:id="rId19"/>
+    <sheet name="ImpactOfCapacityExpansion " sheetId="32" r:id="rId20"/>
+    <sheet name="TotalLifecycleGHGs" sheetId="39" r:id="rId21"/>
+    <sheet name="SocialCostCarbon" sheetId="40" r:id="rId22"/>
   </sheets>
-  <calcPr calcId="191029" iterate="1" iterateDelta="1.0000000000000001E-5"/>
+  <calcPr calcId="191029" refMode="R1C1" iterateCount="0" calcOnSave="0" concurrentCalc="0"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -53,7 +54,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="526" uniqueCount="236">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="532" uniqueCount="242">
   <si>
     <t>category</t>
   </si>
@@ -761,6 +762,24 @@
   </si>
   <si>
     <t>Rural / Non-Council</t>
+  </si>
+  <si>
+    <t>Average of Fuel Economy Combined (kWh/100 mi)</t>
+  </si>
+  <si>
+    <t>Light-Duty</t>
+  </si>
+  <si>
+    <t>Medium-Duty</t>
+  </si>
+  <si>
+    <t>Heavy-Duty</t>
+  </si>
+  <si>
+    <t>Vehicle Type</t>
+  </si>
+  <si>
+    <t>Fuel Efficiency (Wh/mi)</t>
   </si>
 </sst>
 </file>
@@ -2004,6 +2023,109 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
+  <dimension ref="A1:C8"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="30.85546875" customWidth="1"/>
+    <col min="2" max="2" width="27.28515625" customWidth="1"/>
+    <col min="3" max="3" width="24.5703125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>37</v>
+      </c>
+      <c r="B2">
+        <v>13.2</v>
+      </c>
+      <c r="C2">
+        <v>0.62</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>38</v>
+      </c>
+      <c r="B3">
+        <v>16.3</v>
+      </c>
+      <c r="C3">
+        <v>0.70499999999999996</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>39</v>
+      </c>
+      <c r="B4">
+        <v>38.799999999999997</v>
+      </c>
+      <c r="C4">
+        <v>0.86699999999999999</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>40</v>
+      </c>
+      <c r="B5">
+        <v>12.5</v>
+      </c>
+      <c r="C5">
+        <v>0.62</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>41</v>
+      </c>
+      <c r="B6">
+        <v>11.4</v>
+      </c>
+      <c r="C6">
+        <v>0.68500000000000005</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>42</v>
+      </c>
+      <c r="B7">
+        <v>9.1</v>
+      </c>
+      <c r="C7">
+        <v>0.62</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>43</v>
+      </c>
+      <c r="B8">
+        <v>9.1999999999999993</v>
+      </c>
+      <c r="C8">
+        <v>0.62</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{78DDE928-5E41-4857-9D51-91BD8EEB412E}">
   <dimension ref="A1:J15"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2496,7 +2618,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0B00-000000000000}">
   <dimension ref="A1:B7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2565,7 +2687,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0D00-000000000000}">
   <dimension ref="A1:F3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2626,7 +2748,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0E00-000000000000}">
   <dimension ref="A1:D5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2706,7 +2828,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1200-000000000000}">
   <dimension ref="A1:E3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2767,7 +2889,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1300-000000000000}">
   <dimension ref="A1:C6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2848,7 +2970,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1500-000000000000}">
   <dimension ref="A1:D10"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2989,7 +3111,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1600-000000000000}">
   <dimension ref="A1:C5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -3054,7 +3176,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1B00-000000000000}">
   <dimension ref="A1:E12"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -3243,240 +3365,6 @@
       </c>
       <c r="E12">
         <v>1.1499999999999999</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1F00-000000000000}">
-  <dimension ref="A1:E13"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="4" max="4" width="27.5703125" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>139</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>140</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>141</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>143</v>
-      </c>
-      <c r="B2" t="s">
-        <v>144</v>
-      </c>
-      <c r="C2" t="s">
-        <v>145</v>
-      </c>
-      <c r="D2" t="s">
-        <v>146</v>
-      </c>
-      <c r="E2" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>148</v>
-      </c>
-      <c r="B3" t="s">
-        <v>149</v>
-      </c>
-      <c r="C3" t="s">
-        <v>150</v>
-      </c>
-      <c r="D3" t="s">
-        <v>151</v>
-      </c>
-      <c r="E3" t="s">
-        <v>152</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>153</v>
-      </c>
-      <c r="B4" t="s">
-        <v>154</v>
-      </c>
-      <c r="C4" t="s">
-        <v>155</v>
-      </c>
-      <c r="D4" t="s">
-        <v>185</v>
-      </c>
-      <c r="E4">
-        <v>0.1</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>153</v>
-      </c>
-      <c r="B5" t="s">
-        <v>154</v>
-      </c>
-      <c r="C5" t="s">
-        <v>155</v>
-      </c>
-      <c r="D5" t="s">
-        <v>146</v>
-      </c>
-      <c r="E5">
-        <v>0.39</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>156</v>
-      </c>
-      <c r="B6" t="s">
-        <v>157</v>
-      </c>
-      <c r="C6" t="s">
-        <v>158</v>
-      </c>
-      <c r="D6" t="s">
-        <v>185</v>
-      </c>
-      <c r="E6">
-        <v>0.59</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>156</v>
-      </c>
-      <c r="B7" t="s">
-        <v>157</v>
-      </c>
-      <c r="C7" t="s">
-        <v>158</v>
-      </c>
-      <c r="D7" t="s">
-        <v>186</v>
-      </c>
-      <c r="E7">
-        <v>0.79</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>159</v>
-      </c>
-      <c r="B8" t="s">
-        <v>160</v>
-      </c>
-      <c r="C8" t="s">
-        <v>161</v>
-      </c>
-      <c r="D8" t="s">
-        <v>185</v>
-      </c>
-      <c r="E8" t="s">
-        <v>187</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>159</v>
-      </c>
-      <c r="B9" t="s">
-        <v>160</v>
-      </c>
-      <c r="C9" t="s">
-        <v>161</v>
-      </c>
-      <c r="D9" t="s">
-        <v>146</v>
-      </c>
-      <c r="E9" t="s">
-        <v>188</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>162</v>
-      </c>
-      <c r="B10" t="s">
-        <v>163</v>
-      </c>
-      <c r="C10" t="s">
-        <v>164</v>
-      </c>
-      <c r="D10" t="s">
-        <v>185</v>
-      </c>
-      <c r="E10">
-        <v>0.28000000000000003</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>162</v>
-      </c>
-      <c r="B11" t="s">
-        <v>163</v>
-      </c>
-      <c r="C11" t="s">
-        <v>164</v>
-      </c>
-      <c r="D11" t="s">
-        <v>146</v>
-      </c>
-      <c r="E11">
-        <v>0.9</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
-        <v>165</v>
-      </c>
-      <c r="B12" t="s">
-        <v>157</v>
-      </c>
-      <c r="C12" t="s">
-        <v>166</v>
-      </c>
-      <c r="D12" t="s">
-        <v>185</v>
-      </c>
-      <c r="E12">
-        <v>0.2</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>165</v>
-      </c>
-      <c r="B13" t="s">
-        <v>157</v>
-      </c>
-      <c r="C13" t="s">
-        <v>166</v>
-      </c>
-      <c r="D13" t="s">
-        <v>146</v>
-      </c>
-      <c r="E13" t="s">
-        <v>189</v>
       </c>
     </row>
   </sheetData>
@@ -3587,6 +3475,240 @@
 </file>
 
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1F00-000000000000}">
+  <dimension ref="A1:E13"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="4" max="4" width="27.5703125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>141</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>143</v>
+      </c>
+      <c r="B2" t="s">
+        <v>144</v>
+      </c>
+      <c r="C2" t="s">
+        <v>145</v>
+      </c>
+      <c r="D2" t="s">
+        <v>146</v>
+      </c>
+      <c r="E2" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>148</v>
+      </c>
+      <c r="B3" t="s">
+        <v>149</v>
+      </c>
+      <c r="C3" t="s">
+        <v>150</v>
+      </c>
+      <c r="D3" t="s">
+        <v>151</v>
+      </c>
+      <c r="E3" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>153</v>
+      </c>
+      <c r="B4" t="s">
+        <v>154</v>
+      </c>
+      <c r="C4" t="s">
+        <v>155</v>
+      </c>
+      <c r="D4" t="s">
+        <v>185</v>
+      </c>
+      <c r="E4">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>153</v>
+      </c>
+      <c r="B5" t="s">
+        <v>154</v>
+      </c>
+      <c r="C5" t="s">
+        <v>155</v>
+      </c>
+      <c r="D5" t="s">
+        <v>146</v>
+      </c>
+      <c r="E5">
+        <v>0.39</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>156</v>
+      </c>
+      <c r="B6" t="s">
+        <v>157</v>
+      </c>
+      <c r="C6" t="s">
+        <v>158</v>
+      </c>
+      <c r="D6" t="s">
+        <v>185</v>
+      </c>
+      <c r="E6">
+        <v>0.59</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>156</v>
+      </c>
+      <c r="B7" t="s">
+        <v>157</v>
+      </c>
+      <c r="C7" t="s">
+        <v>158</v>
+      </c>
+      <c r="D7" t="s">
+        <v>186</v>
+      </c>
+      <c r="E7">
+        <v>0.79</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>159</v>
+      </c>
+      <c r="B8" t="s">
+        <v>160</v>
+      </c>
+      <c r="C8" t="s">
+        <v>161</v>
+      </c>
+      <c r="D8" t="s">
+        <v>185</v>
+      </c>
+      <c r="E8" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>159</v>
+      </c>
+      <c r="B9" t="s">
+        <v>160</v>
+      </c>
+      <c r="C9" t="s">
+        <v>161</v>
+      </c>
+      <c r="D9" t="s">
+        <v>146</v>
+      </c>
+      <c r="E9" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>162</v>
+      </c>
+      <c r="B10" t="s">
+        <v>163</v>
+      </c>
+      <c r="C10" t="s">
+        <v>164</v>
+      </c>
+      <c r="D10" t="s">
+        <v>185</v>
+      </c>
+      <c r="E10">
+        <v>0.28000000000000003</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>162</v>
+      </c>
+      <c r="B11" t="s">
+        <v>163</v>
+      </c>
+      <c r="C11" t="s">
+        <v>164</v>
+      </c>
+      <c r="D11" t="s">
+        <v>146</v>
+      </c>
+      <c r="E11">
+        <v>0.9</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>165</v>
+      </c>
+      <c r="B12" t="s">
+        <v>157</v>
+      </c>
+      <c r="C12" t="s">
+        <v>166</v>
+      </c>
+      <c r="D12" t="s">
+        <v>185</v>
+      </c>
+      <c r="E12">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>165</v>
+      </c>
+      <c r="B13" t="s">
+        <v>157</v>
+      </c>
+      <c r="C13" t="s">
+        <v>166</v>
+      </c>
+      <c r="D13" t="s">
+        <v>146</v>
+      </c>
+      <c r="E13" t="s">
+        <v>189</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-2600-000000000000}">
   <dimension ref="A1:E7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -3716,7 +3838,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FC06F369-1B95-458E-A555-6CC2EF2B1D77}">
   <dimension ref="A1:E184"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -7654,6 +7776,64 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9826AB9F-6D6F-4C88-8814-100BD402A958}">
+  <dimension ref="A1:C4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="16" customWidth="1"/>
+    <col min="2" max="2" width="40.42578125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>240</v>
+      </c>
+      <c r="B1" t="s">
+        <v>236</v>
+      </c>
+      <c r="C1" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>237</v>
+      </c>
+      <c r="B2">
+        <v>37.844029636270804</v>
+      </c>
+      <c r="C2">
+        <v>2642.4247354504005</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>238</v>
+      </c>
+      <c r="B3">
+        <v>145.51450894247785</v>
+      </c>
+      <c r="C3">
+        <v>687.21669561851172</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>239</v>
+      </c>
+      <c r="B4">
+        <v>158.85714285714286</v>
+      </c>
+      <c r="C4">
+        <v>629.49640287769785</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:D8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -7775,7 +7955,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:D5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -7855,7 +8035,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <dimension ref="A1:D6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -7930,107 +8110,4 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
-  <dimension ref="A1:C8"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="30.85546875" customWidth="1"/>
-    <col min="2" max="2" width="27.28515625" customWidth="1"/>
-    <col min="3" max="3" width="24.5703125" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>37</v>
-      </c>
-      <c r="B2">
-        <v>13.2</v>
-      </c>
-      <c r="C2">
-        <v>0.62</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>38</v>
-      </c>
-      <c r="B3">
-        <v>16.3</v>
-      </c>
-      <c r="C3">
-        <v>0.70499999999999996</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>39</v>
-      </c>
-      <c r="B4">
-        <v>38.799999999999997</v>
-      </c>
-      <c r="C4">
-        <v>0.86699999999999999</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>40</v>
-      </c>
-      <c r="B5">
-        <v>12.5</v>
-      </c>
-      <c r="C5">
-        <v>0.62</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>41</v>
-      </c>
-      <c r="B6">
-        <v>11.4</v>
-      </c>
-      <c r="C6">
-        <v>0.68500000000000005</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>42</v>
-      </c>
-      <c r="B7">
-        <v>9.1</v>
-      </c>
-      <c r="C7">
-        <v>0.62</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>43</v>
-      </c>
-      <c r="B8">
-        <v>9.1999999999999993</v>
-      </c>
-      <c r="C8">
-        <v>0.62</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
finishing up pedestrian facilities
</commit_message>
<xml_diff>
--- a/data/MetCouncilTables.xlsx
+++ b/data/MetCouncilTables.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://icfonline-my.sharepoint.com/personal/61886_icf_com/Documents/Desktop/transport-emission-shiny/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="167" documentId="8_{BBC49CD7-68E0-4D8F-B576-EE14E509F0DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{55D89571-C465-45CA-8F78-FAE742371238}"/>
+  <xr:revisionPtr revIDLastSave="172" documentId="8_{BBC49CD7-68E0-4D8F-B576-EE14E509F0DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0EEFC7CE-AED0-4FF9-A1D8-8789AC8500D9}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="14310" windowHeight="15480" firstSheet="5" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-60" yWindow="45" windowWidth="22710" windowHeight="15585" firstSheet="13" activeTab="16" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="TripDistances" sheetId="42" r:id="rId1"/>
@@ -36,7 +36,7 @@
     <sheet name="TotalLifecycleGHGs" sheetId="39" r:id="rId21"/>
     <sheet name="SocialCostCarbon" sheetId="40" r:id="rId22"/>
   </sheets>
-  <calcPr calcId="191029" refMode="R1C1" iterateCount="0" calcOnSave="0" concurrentCalc="0"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -54,7 +54,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="532" uniqueCount="242">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="531" uniqueCount="241">
   <si>
     <t>category</t>
   </si>
@@ -600,9 +600,6 @@
   </si>
   <si>
     <t>one_way_facility_length_miles_low</t>
-  </si>
-  <si>
-    <t>one_way_facility_length_miles_high</t>
   </si>
   <si>
     <t>idling_fuel_use_gal_hr_no_load</t>
@@ -1629,33 +1626,33 @@
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>199</v>
+      </c>
+      <c r="B1" t="s">
         <v>200</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>201</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>202</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>203</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>204</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>205</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>206</v>
-      </c>
-      <c r="H1" t="s">
-        <v>207</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="B2">
         <v>2.9749119231916001</v>
@@ -1681,7 +1678,7 @@
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="B3">
         <v>3.6999170502861798</v>
@@ -1699,7 +1696,7 @@
         <v>4.2547154693920097</v>
       </c>
       <c r="G3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="H3">
         <v>30</v>
@@ -1707,7 +1704,7 @@
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="B4">
         <v>5.9016230035503296</v>
@@ -1733,7 +1730,7 @@
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="B5">
         <v>3.8634645109851302</v>
@@ -1748,10 +1745,10 @@
         <v>3.8634645109851302</v>
       </c>
       <c r="F5" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="G5" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="H5">
         <v>1</v>
@@ -1759,7 +1756,7 @@
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="B6">
         <v>0.71198948216291502</v>
@@ -1785,7 +1782,7 @@
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="B7">
         <v>0.97570910188785598</v>
@@ -1811,7 +1808,7 @@
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="B8">
         <v>6.4778152091502204</v>
@@ -1837,7 +1834,7 @@
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="B9">
         <v>7.7004599845074297</v>
@@ -1863,7 +1860,7 @@
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="B10">
         <v>5.8322002863550404</v>
@@ -1889,7 +1886,7 @@
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="B11">
         <v>5.2559515730838502</v>
@@ -1915,7 +1912,7 @@
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="B12">
         <v>4.3043541561638703</v>
@@ -1941,7 +1938,7 @@
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="B13">
         <v>4.4554427783066402</v>
@@ -1967,7 +1964,7 @@
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="B14">
         <v>5.8745743082736501</v>
@@ -1993,7 +1990,7 @@
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="B15">
         <v>0.85801128591603704</v>
@@ -2135,34 +2132,34 @@
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>222</v>
+      </c>
+      <c r="B1" t="s">
         <v>223</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>224</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>225</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>226</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>227</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>228</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
+        <v>206</v>
+      </c>
+      <c r="I1" t="s">
         <v>229</v>
       </c>
-      <c r="H1" t="s">
-        <v>207</v>
-      </c>
-      <c r="I1" t="s">
+      <c r="J1" t="s">
         <v>230</v>
-      </c>
-      <c r="J1" t="s">
-        <v>231</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
@@ -2194,7 +2191,7 @@
         <v>2040</v>
       </c>
       <c r="J2" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.25">
@@ -2226,7 +2223,7 @@
         <v>2040</v>
       </c>
       <c r="J3" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.25">
@@ -2258,7 +2255,7 @@
         <v>2040</v>
       </c>
       <c r="J4" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.25">
@@ -2290,7 +2287,7 @@
         <v>2040</v>
       </c>
       <c r="J5" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.25">
@@ -2322,7 +2319,7 @@
         <v>2040</v>
       </c>
       <c r="J6" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.25">
@@ -2354,7 +2351,7 @@
         <v>2040</v>
       </c>
       <c r="J7" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.25">
@@ -2386,7 +2383,7 @@
         <v>2040</v>
       </c>
       <c r="J8" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.25">
@@ -2418,7 +2415,7 @@
         <v>2040</v>
       </c>
       <c r="J9" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.25">
@@ -2450,7 +2447,7 @@
         <v>2050</v>
       </c>
       <c r="J10" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.25">
@@ -2482,7 +2479,7 @@
         <v>2050</v>
       </c>
       <c r="J11" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.25">
@@ -2514,7 +2511,7 @@
         <v>2050</v>
       </c>
       <c r="J12" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.25">
@@ -2546,7 +2543,7 @@
         <v>2050</v>
       </c>
       <c r="J13" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.25">
@@ -2578,7 +2575,7 @@
         <v>2050</v>
       </c>
       <c r="J14" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.25">
@@ -2610,7 +2607,7 @@
         <v>2050</v>
       </c>
       <c r="J15" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
     </row>
   </sheetData>
@@ -2972,10 +2969,15 @@
 
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1500-000000000000}">
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:C10"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="22" customWidth="1"/>
+    <col min="2" max="2" width="35.5703125" customWidth="1"/>
+    <col min="3" max="3" width="47.85546875" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>112</v>
       </c>
@@ -2983,13 +2985,10 @@
         <v>181</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>182</v>
-      </c>
-      <c r="D1" s="1" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>114</v>
       </c>
@@ -2997,13 +2996,10 @@
         <v>1</v>
       </c>
       <c r="C2">
-        <v>1</v>
-      </c>
-      <c r="D2">
         <v>1.9E-3</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>114</v>
       </c>
@@ -3011,24 +3007,21 @@
         <v>1.01</v>
       </c>
       <c r="C3">
-        <v>2</v>
-      </c>
-      <c r="D3">
         <v>2.8999999999999998E-3</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>114</v>
       </c>
       <c r="B4">
         <v>2</v>
       </c>
-      <c r="D4">
+      <c r="C4">
         <v>3.8E-3</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>115</v>
       </c>
@@ -3036,13 +3029,10 @@
         <v>1</v>
       </c>
       <c r="C5">
-        <v>1</v>
-      </c>
-      <c r="D5">
         <v>1.4E-3</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>115</v>
       </c>
@@ -3050,24 +3040,21 @@
         <v>1.01</v>
       </c>
       <c r="C6">
-        <v>2</v>
-      </c>
-      <c r="D6">
         <v>2E-3</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>115</v>
       </c>
       <c r="B7">
         <v>2</v>
       </c>
-      <c r="D7">
+      <c r="C7">
         <v>2.7000000000000001E-3</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>116</v>
       </c>
@@ -3075,13 +3062,10 @@
         <v>1</v>
       </c>
       <c r="C8">
-        <v>1</v>
-      </c>
-      <c r="D8">
         <v>1E-3</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>116</v>
       </c>
@@ -3089,20 +3073,17 @@
         <v>1.01</v>
       </c>
       <c r="C9">
-        <v>2</v>
-      </c>
-      <c r="D9">
         <v>1.4E-3</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>116</v>
       </c>
       <c r="B10">
         <v>2</v>
       </c>
-      <c r="D10">
+      <c r="C10">
         <v>1.9E-3</v>
       </c>
     </row>
@@ -3195,10 +3176,10 @@
         <v>125</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>182</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>183</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>184</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
@@ -3544,7 +3525,7 @@
         <v>155</v>
       </c>
       <c r="D4" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="E4">
         <v>0.1</v>
@@ -3578,7 +3559,7 @@
         <v>158</v>
       </c>
       <c r="D6" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="E6">
         <v>0.59</v>
@@ -3595,7 +3576,7 @@
         <v>158</v>
       </c>
       <c r="D7" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="E7">
         <v>0.79</v>
@@ -3612,10 +3593,10 @@
         <v>161</v>
       </c>
       <c r="D8" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="E8" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
@@ -3632,7 +3613,7 @@
         <v>146</v>
       </c>
       <c r="E9" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
@@ -3646,7 +3627,7 @@
         <v>164</v>
       </c>
       <c r="D10" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="E10">
         <v>0.28000000000000003</v>
@@ -3680,7 +3661,7 @@
         <v>166</v>
       </c>
       <c r="D12" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="E12">
         <v>0.2</v>
@@ -3700,7 +3681,7 @@
         <v>146</v>
       </c>
       <c r="E13" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
     </row>
   </sheetData>
@@ -3722,7 +3703,7 @@
   <sheetData>
     <row r="1" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>167</v>
@@ -3845,24 +3826,24 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>190</v>
+      </c>
+      <c r="B1" t="s">
         <v>191</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>192</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>193</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>194</v>
-      </c>
-      <c r="E1" t="s">
-        <v>195</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="B2">
         <v>2020</v>
@@ -3879,7 +3860,7 @@
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="B3">
         <v>2021</v>
@@ -3896,7 +3877,7 @@
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="B4">
         <v>2022</v>
@@ -3913,7 +3894,7 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="B5">
         <v>2023</v>
@@ -3930,7 +3911,7 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="B6">
         <v>2024</v>
@@ -3947,7 +3928,7 @@
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="B7">
         <v>2025</v>
@@ -3964,7 +3945,7 @@
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="B8">
         <v>2026</v>
@@ -3981,7 +3962,7 @@
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="B9">
         <v>2027</v>
@@ -3998,7 +3979,7 @@
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="B10">
         <v>2028</v>
@@ -4015,7 +3996,7 @@
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="B11">
         <v>2029</v>
@@ -4032,7 +4013,7 @@
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="B12">
         <v>2030</v>
@@ -4049,7 +4030,7 @@
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="B13">
         <v>2031</v>
@@ -4066,7 +4047,7 @@
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="B14">
         <v>2032</v>
@@ -4083,7 +4064,7 @@
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="B15">
         <v>2033</v>
@@ -4100,7 +4081,7 @@
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="B16">
         <v>2034</v>
@@ -4117,7 +4098,7 @@
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="B17">
         <v>2035</v>
@@ -4134,7 +4115,7 @@
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="B18">
         <v>2036</v>
@@ -4151,7 +4132,7 @@
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="B19">
         <v>2037</v>
@@ -4168,7 +4149,7 @@
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="B20">
         <v>2038</v>
@@ -4185,7 +4166,7 @@
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="B21">
         <v>2039</v>
@@ -4202,7 +4183,7 @@
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="B22">
         <v>2040</v>
@@ -4219,7 +4200,7 @@
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="B23">
         <v>2041</v>
@@ -4236,7 +4217,7 @@
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="B24">
         <v>2042</v>
@@ -4253,7 +4234,7 @@
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="B25">
         <v>2043</v>
@@ -4270,7 +4251,7 @@
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="B26">
         <v>2044</v>
@@ -4287,7 +4268,7 @@
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="B27">
         <v>2045</v>
@@ -4304,7 +4285,7 @@
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="B28">
         <v>2046</v>
@@ -4321,7 +4302,7 @@
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="B29">
         <v>2047</v>
@@ -4338,7 +4319,7 @@
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="B30">
         <v>2048</v>
@@ -4355,7 +4336,7 @@
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="B31">
         <v>2049</v>
@@ -4372,7 +4353,7 @@
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="B32">
         <v>2050</v>
@@ -4389,7 +4370,7 @@
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="B33">
         <v>2051</v>
@@ -4406,7 +4387,7 @@
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="B34">
         <v>2052</v>
@@ -4423,7 +4404,7 @@
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="B35">
         <v>2053</v>
@@ -4440,7 +4421,7 @@
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="B36">
         <v>2054</v>
@@ -4457,7 +4438,7 @@
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="B37">
         <v>2055</v>
@@ -4474,7 +4455,7 @@
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="B38">
         <v>2056</v>
@@ -4491,7 +4472,7 @@
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="B39">
         <v>2057</v>
@@ -4508,7 +4489,7 @@
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="B40">
         <v>2058</v>
@@ -4525,7 +4506,7 @@
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="B41">
         <v>2059</v>
@@ -4542,7 +4523,7 @@
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="B42">
         <v>2060</v>
@@ -4559,7 +4540,7 @@
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="B43">
         <v>2061</v>
@@ -4576,7 +4557,7 @@
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="B44">
         <v>2062</v>
@@ -4593,7 +4574,7 @@
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="B45">
         <v>2063</v>
@@ -4610,7 +4591,7 @@
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="B46">
         <v>2064</v>
@@ -4627,7 +4608,7 @@
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="B47">
         <v>2065</v>
@@ -4644,7 +4625,7 @@
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="B48">
         <v>2066</v>
@@ -4661,7 +4642,7 @@
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="B49">
         <v>2067</v>
@@ -4678,7 +4659,7 @@
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="B50">
         <v>2068</v>
@@ -4695,7 +4676,7 @@
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="B51">
         <v>2069</v>
@@ -4712,7 +4693,7 @@
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="B52">
         <v>2070</v>
@@ -4729,7 +4710,7 @@
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="B53">
         <v>2071</v>
@@ -4746,7 +4727,7 @@
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="B54">
         <v>2072</v>
@@ -4763,7 +4744,7 @@
     </row>
     <row r="55" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="B55">
         <v>2073</v>
@@ -4780,7 +4761,7 @@
     </row>
     <row r="56" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="B56">
         <v>2074</v>
@@ -4797,7 +4778,7 @@
     </row>
     <row r="57" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="B57">
         <v>2075</v>
@@ -4814,7 +4795,7 @@
     </row>
     <row r="58" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="B58">
         <v>2076</v>
@@ -4831,7 +4812,7 @@
     </row>
     <row r="59" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="B59">
         <v>2077</v>
@@ -4848,7 +4829,7 @@
     </row>
     <row r="60" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="B60">
         <v>2078</v>
@@ -4865,7 +4846,7 @@
     </row>
     <row r="61" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="B61">
         <v>2079</v>
@@ -4882,7 +4863,7 @@
     </row>
     <row r="62" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="B62">
         <v>2080</v>
@@ -4899,7 +4880,7 @@
     </row>
     <row r="63" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B63">
         <v>2020</v>
@@ -4916,7 +4897,7 @@
     </row>
     <row r="64" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B64">
         <v>2021</v>
@@ -4933,7 +4914,7 @@
     </row>
     <row r="65" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B65">
         <v>2022</v>
@@ -4950,7 +4931,7 @@
     </row>
     <row r="66" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B66">
         <v>2023</v>
@@ -4967,7 +4948,7 @@
     </row>
     <row r="67" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B67">
         <v>2024</v>
@@ -4984,7 +4965,7 @@
     </row>
     <row r="68" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B68">
         <v>2025</v>
@@ -5001,7 +4982,7 @@
     </row>
     <row r="69" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B69">
         <v>2026</v>
@@ -5018,7 +4999,7 @@
     </row>
     <row r="70" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B70">
         <v>2027</v>
@@ -5035,7 +5016,7 @@
     </row>
     <row r="71" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B71">
         <v>2028</v>
@@ -5052,7 +5033,7 @@
     </row>
     <row r="72" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B72">
         <v>2029</v>
@@ -5069,7 +5050,7 @@
     </row>
     <row r="73" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B73">
         <v>2030</v>
@@ -5086,7 +5067,7 @@
     </row>
     <row r="74" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B74">
         <v>2031</v>
@@ -5103,7 +5084,7 @@
     </row>
     <row r="75" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B75">
         <v>2032</v>
@@ -5120,7 +5101,7 @@
     </row>
     <row r="76" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B76">
         <v>2033</v>
@@ -5137,7 +5118,7 @@
     </row>
     <row r="77" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B77">
         <v>2034</v>
@@ -5154,7 +5135,7 @@
     </row>
     <row r="78" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B78">
         <v>2035</v>
@@ -5171,7 +5152,7 @@
     </row>
     <row r="79" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B79">
         <v>2036</v>
@@ -5188,7 +5169,7 @@
     </row>
     <row r="80" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B80">
         <v>2037</v>
@@ -5205,7 +5186,7 @@
     </row>
     <row r="81" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B81">
         <v>2038</v>
@@ -5222,7 +5203,7 @@
     </row>
     <row r="82" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B82">
         <v>2039</v>
@@ -5239,7 +5220,7 @@
     </row>
     <row r="83" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B83">
         <v>2040</v>
@@ -5256,7 +5237,7 @@
     </row>
     <row r="84" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B84">
         <v>2041</v>
@@ -5273,7 +5254,7 @@
     </row>
     <row r="85" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B85">
         <v>2042</v>
@@ -5290,7 +5271,7 @@
     </row>
     <row r="86" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B86">
         <v>2043</v>
@@ -5307,7 +5288,7 @@
     </row>
     <row r="87" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B87">
         <v>2044</v>
@@ -5324,7 +5305,7 @@
     </row>
     <row r="88" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B88">
         <v>2045</v>
@@ -5341,7 +5322,7 @@
     </row>
     <row r="89" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B89">
         <v>2046</v>
@@ -5358,7 +5339,7 @@
     </row>
     <row r="90" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B90">
         <v>2047</v>
@@ -5375,7 +5356,7 @@
     </row>
     <row r="91" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B91">
         <v>2048</v>
@@ -5392,7 +5373,7 @@
     </row>
     <row r="92" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B92">
         <v>2049</v>
@@ -5409,7 +5390,7 @@
     </row>
     <row r="93" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B93">
         <v>2050</v>
@@ -5426,7 +5407,7 @@
     </row>
     <row r="94" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B94">
         <v>2051</v>
@@ -5443,7 +5424,7 @@
     </row>
     <row r="95" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B95">
         <v>2052</v>
@@ -5460,7 +5441,7 @@
     </row>
     <row r="96" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B96">
         <v>2053</v>
@@ -5477,7 +5458,7 @@
     </row>
     <row r="97" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B97">
         <v>2054</v>
@@ -5494,7 +5475,7 @@
     </row>
     <row r="98" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B98">
         <v>2055</v>
@@ -5511,7 +5492,7 @@
     </row>
     <row r="99" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B99">
         <v>2056</v>
@@ -5528,7 +5509,7 @@
     </row>
     <row r="100" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B100">
         <v>2057</v>
@@ -5545,7 +5526,7 @@
     </row>
     <row r="101" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B101">
         <v>2058</v>
@@ -5562,7 +5543,7 @@
     </row>
     <row r="102" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B102">
         <v>2059</v>
@@ -5579,7 +5560,7 @@
     </row>
     <row r="103" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B103">
         <v>2060</v>
@@ -5596,7 +5577,7 @@
     </row>
     <row r="104" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B104">
         <v>2061</v>
@@ -5613,7 +5594,7 @@
     </row>
     <row r="105" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B105">
         <v>2062</v>
@@ -5630,7 +5611,7 @@
     </row>
     <row r="106" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B106">
         <v>2063</v>
@@ -5647,7 +5628,7 @@
     </row>
     <row r="107" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B107">
         <v>2064</v>
@@ -5664,7 +5645,7 @@
     </row>
     <row r="108" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B108">
         <v>2065</v>
@@ -5681,7 +5662,7 @@
     </row>
     <row r="109" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B109">
         <v>2066</v>
@@ -5698,7 +5679,7 @@
     </row>
     <row r="110" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B110">
         <v>2067</v>
@@ -5715,7 +5696,7 @@
     </row>
     <row r="111" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B111">
         <v>2068</v>
@@ -5732,7 +5713,7 @@
     </row>
     <row r="112" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A112" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B112">
         <v>2069</v>
@@ -5749,7 +5730,7 @@
     </row>
     <row r="113" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A113" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B113">
         <v>2070</v>
@@ -5766,7 +5747,7 @@
     </row>
     <row r="114" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A114" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B114">
         <v>2071</v>
@@ -5783,7 +5764,7 @@
     </row>
     <row r="115" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A115" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B115">
         <v>2072</v>
@@ -5800,7 +5781,7 @@
     </row>
     <row r="116" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A116" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B116">
         <v>2073</v>
@@ -5817,7 +5798,7 @@
     </row>
     <row r="117" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A117" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B117">
         <v>2074</v>
@@ -5834,7 +5815,7 @@
     </row>
     <row r="118" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A118" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B118">
         <v>2075</v>
@@ -5851,7 +5832,7 @@
     </row>
     <row r="119" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A119" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B119">
         <v>2076</v>
@@ -5868,7 +5849,7 @@
     </row>
     <row r="120" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A120" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B120">
         <v>2077</v>
@@ -5885,7 +5866,7 @@
     </row>
     <row r="121" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A121" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B121">
         <v>2078</v>
@@ -5902,7 +5883,7 @@
     </row>
     <row r="122" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A122" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B122">
         <v>2079</v>
@@ -5919,7 +5900,7 @@
     </row>
     <row r="123" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A123" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B123">
         <v>2080</v>
@@ -5936,7 +5917,7 @@
     </row>
     <row r="124" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A124" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B124">
         <v>2020</v>
@@ -5953,7 +5934,7 @@
     </row>
     <row r="125" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A125" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B125">
         <v>2021</v>
@@ -5970,7 +5951,7 @@
     </row>
     <row r="126" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A126" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B126">
         <v>2022</v>
@@ -5987,7 +5968,7 @@
     </row>
     <row r="127" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A127" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B127">
         <v>2023</v>
@@ -6004,7 +5985,7 @@
     </row>
     <row r="128" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A128" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B128">
         <v>2024</v>
@@ -6021,7 +6002,7 @@
     </row>
     <row r="129" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A129" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B129">
         <v>2025</v>
@@ -6038,7 +6019,7 @@
     </row>
     <row r="130" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A130" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B130">
         <v>2026</v>
@@ -6055,7 +6036,7 @@
     </row>
     <row r="131" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A131" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B131">
         <v>2027</v>
@@ -6072,7 +6053,7 @@
     </row>
     <row r="132" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A132" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B132">
         <v>2028</v>
@@ -6089,7 +6070,7 @@
     </row>
     <row r="133" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A133" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B133">
         <v>2029</v>
@@ -6106,7 +6087,7 @@
     </row>
     <row r="134" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A134" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B134">
         <v>2030</v>
@@ -6123,7 +6104,7 @@
     </row>
     <row r="135" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A135" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B135">
         <v>2031</v>
@@ -6140,7 +6121,7 @@
     </row>
     <row r="136" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A136" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B136">
         <v>2032</v>
@@ -6157,7 +6138,7 @@
     </row>
     <row r="137" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A137" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B137">
         <v>2033</v>
@@ -6174,7 +6155,7 @@
     </row>
     <row r="138" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A138" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B138">
         <v>2034</v>
@@ -6191,7 +6172,7 @@
     </row>
     <row r="139" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A139" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B139">
         <v>2035</v>
@@ -6208,7 +6189,7 @@
     </row>
     <row r="140" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A140" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B140">
         <v>2036</v>
@@ -6225,7 +6206,7 @@
     </row>
     <row r="141" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A141" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B141">
         <v>2037</v>
@@ -6242,7 +6223,7 @@
     </row>
     <row r="142" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A142" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B142">
         <v>2038</v>
@@ -6259,7 +6240,7 @@
     </row>
     <row r="143" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A143" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B143">
         <v>2039</v>
@@ -6276,7 +6257,7 @@
     </row>
     <row r="144" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A144" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B144">
         <v>2040</v>
@@ -6293,7 +6274,7 @@
     </row>
     <row r="145" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A145" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B145">
         <v>2041</v>
@@ -6310,7 +6291,7 @@
     </row>
     <row r="146" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A146" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B146">
         <v>2042</v>
@@ -6327,7 +6308,7 @@
     </row>
     <row r="147" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A147" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B147">
         <v>2043</v>
@@ -6344,7 +6325,7 @@
     </row>
     <row r="148" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A148" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B148">
         <v>2044</v>
@@ -6361,7 +6342,7 @@
     </row>
     <row r="149" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A149" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B149">
         <v>2045</v>
@@ -6378,7 +6359,7 @@
     </row>
     <row r="150" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A150" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B150">
         <v>2046</v>
@@ -6395,7 +6376,7 @@
     </row>
     <row r="151" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A151" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B151">
         <v>2047</v>
@@ -6412,7 +6393,7 @@
     </row>
     <row r="152" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A152" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B152">
         <v>2048</v>
@@ -6429,7 +6410,7 @@
     </row>
     <row r="153" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A153" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B153">
         <v>2049</v>
@@ -6446,7 +6427,7 @@
     </row>
     <row r="154" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A154" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B154">
         <v>2050</v>
@@ -6463,7 +6444,7 @@
     </row>
     <row r="155" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A155" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B155">
         <v>2051</v>
@@ -6480,7 +6461,7 @@
     </row>
     <row r="156" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A156" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B156">
         <v>2052</v>
@@ -6497,7 +6478,7 @@
     </row>
     <row r="157" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A157" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B157">
         <v>2053</v>
@@ -6514,7 +6495,7 @@
     </row>
     <row r="158" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A158" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B158">
         <v>2054</v>
@@ -6531,7 +6512,7 @@
     </row>
     <row r="159" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A159" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B159">
         <v>2055</v>
@@ -6548,7 +6529,7 @@
     </row>
     <row r="160" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A160" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B160">
         <v>2056</v>
@@ -6565,7 +6546,7 @@
     </row>
     <row r="161" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A161" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B161">
         <v>2057</v>
@@ -6582,7 +6563,7 @@
     </row>
     <row r="162" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A162" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B162">
         <v>2058</v>
@@ -6599,7 +6580,7 @@
     </row>
     <row r="163" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A163" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B163">
         <v>2059</v>
@@ -6616,7 +6597,7 @@
     </row>
     <row r="164" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A164" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B164">
         <v>2060</v>
@@ -6633,7 +6614,7 @@
     </row>
     <row r="165" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A165" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B165">
         <v>2061</v>
@@ -6650,7 +6631,7 @@
     </row>
     <row r="166" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A166" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B166">
         <v>2062</v>
@@ -6667,7 +6648,7 @@
     </row>
     <row r="167" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A167" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B167">
         <v>2063</v>
@@ -6684,7 +6665,7 @@
     </row>
     <row r="168" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A168" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B168">
         <v>2064</v>
@@ -6701,7 +6682,7 @@
     </row>
     <row r="169" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A169" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B169">
         <v>2065</v>
@@ -6718,7 +6699,7 @@
     </row>
     <row r="170" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A170" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B170">
         <v>2066</v>
@@ -6735,7 +6716,7 @@
     </row>
     <row r="171" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A171" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B171">
         <v>2067</v>
@@ -6752,7 +6733,7 @@
     </row>
     <row r="172" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A172" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B172">
         <v>2068</v>
@@ -6769,7 +6750,7 @@
     </row>
     <row r="173" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A173" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B173">
         <v>2069</v>
@@ -6786,7 +6767,7 @@
     </row>
     <row r="174" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A174" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B174">
         <v>2070</v>
@@ -6803,7 +6784,7 @@
     </row>
     <row r="175" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A175" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B175">
         <v>2071</v>
@@ -6820,7 +6801,7 @@
     </row>
     <row r="176" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A176" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B176">
         <v>2072</v>
@@ -6837,7 +6818,7 @@
     </row>
     <row r="177" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A177" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B177">
         <v>2073</v>
@@ -6854,7 +6835,7 @@
     </row>
     <row r="178" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A178" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B178">
         <v>2074</v>
@@ -6871,7 +6852,7 @@
     </row>
     <row r="179" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A179" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B179">
         <v>2075</v>
@@ -6888,7 +6869,7 @@
     </row>
     <row r="180" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A180" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B180">
         <v>2076</v>
@@ -6905,7 +6886,7 @@
     </row>
     <row r="181" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A181" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B181">
         <v>2077</v>
@@ -6922,7 +6903,7 @@
     </row>
     <row r="182" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A182" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B182">
         <v>2078</v>
@@ -6939,7 +6920,7 @@
     </row>
     <row r="183" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A183" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B183">
         <v>2079</v>
@@ -6956,7 +6937,7 @@
     </row>
     <row r="184" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A184" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B184">
         <v>2080</v>
@@ -7185,7 +7166,7 @@
   <sheetData>
     <row r="1" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>44</v>
@@ -7786,18 +7767,18 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>239</v>
+      </c>
+      <c r="B1" t="s">
+        <v>235</v>
+      </c>
+      <c r="C1" t="s">
         <v>240</v>
-      </c>
-      <c r="B1" t="s">
-        <v>236</v>
-      </c>
-      <c r="C1" t="s">
-        <v>241</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="B2">
         <v>37.844029636270804</v>
@@ -7808,7 +7789,7 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="B3">
         <v>145.51450894247785</v>
@@ -7819,7 +7800,7 @@
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="B4">
         <v>158.85714285714286</v>

</xml_diff>

<commit_message>
updated inputs to ev infrastructure, updated EFs, shared mobility and ev outreach factor changes
</commit_message>
<xml_diff>
--- a/data/MetCouncilTables.xlsx
+++ b/data/MetCouncilTables.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://icfonline-my.sharepoint.com/personal/61886_icf_com/Documents/Desktop/transport-emission-shiny/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="315" documentId="8_{BBC49CD7-68E0-4D8F-B576-EE14E509F0DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BA84BD61-C6FF-40F6-8A99-E9DDC49C5F75}"/>
+  <xr:revisionPtr revIDLastSave="324" documentId="8_{BBC49CD7-68E0-4D8F-B576-EE14E509F0DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{09E128ED-54EB-4E76-BB60-88D39D8E86D1}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-3450" windowWidth="29040" windowHeight="15720" firstSheet="9" activeTab="12" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-3450" windowWidth="29040" windowHeight="15720" firstSheet="2" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="TripDistances" sheetId="42" r:id="rId1"/>
@@ -8329,7 +8329,8 @@
         <v>37.844029636270804</v>
       </c>
       <c r="C2">
-        <v>2642.4247354504005</v>
+        <f xml:space="preserve"> B2 * 10</f>
+        <v>378.44029636270807</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -8340,7 +8341,8 @@
         <v>145.51450894247785</v>
       </c>
       <c r="C3">
-        <v>687.21669561851172</v>
+        <f t="shared" ref="C3:C4" si="0" xml:space="preserve"> B3 * 10</f>
+        <v>1455.1450894247785</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
@@ -8351,7 +8353,8 @@
         <v>158.85714285714286</v>
       </c>
       <c r="C4">
-        <v>629.49640287769785</v>
+        <f t="shared" si="0"/>
+        <v>1588.5714285714287</v>
       </c>
     </row>
   </sheetData>

</xml_diff>